<commit_message>
Update Decision_Summary and notes to new node labels
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Measured corner link J-OUEST-AVAL -&gt; J-BASSIN-OUEST</t>
+          <t>Measured corner link P-W6 -&gt; MH-BASSIN-OUEST</t>
         </is>
       </c>
       <c r="D14" s="3" t="n"/>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>J-BASSIN-IN -&gt; BASSIN-RET</t>
+          <t>MH-BASSIN-EST -&gt; BASSIN-RET</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>J-BASSIN-OUEST -&gt; BASSIN-RET</t>
+          <t>MH-BASSIN-OUEST -&gt; RP-02 / bassin path</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
@@ -2270,7 +2270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="145" customWidth="1" style="22" min="1" max="1"/>
@@ -2284,7 +2284,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2348,8 +2347,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
@@ -2651,7 +2648,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="35" t="inlineStr">
         <is>
@@ -2680,24 +2676,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -3546,7 +3524,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Cote plan visible (J-OUEST-AMONT jusqu'a fin zone amont avant troncon pave inferieur).</t>
+          <t>Cote plan visible (P-W1 jusqu'a fin zone amont avant troncon pave inferieur).</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3770,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Distance mesuree J-OUEST-AVAL -&gt; entree ouest bassin (image utilisateur).</t>
+          <t>Distance mesuree P-W6 -&gt; MH-BASSIN-OUEST (image utilisateur).</t>
         </is>
       </c>
     </row>
@@ -11934,7 +11912,7 @@
       </c>
       <c r="AB6" s="3" t="inlineStr">
         <is>
-          <t>Entree EST: P-03 -&gt; J-BASSIN-IN (16.1 m).</t>
+          <t>Entree EST: P-03 -&gt; MH-BASSIN-EST (16.1 m).</t>
         </is>
       </c>
       <c r="AC6" s="8" t="n"/>
@@ -41365,7 +41343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="20" customWidth="1" style="22" min="1" max="1"/>
@@ -41882,29 +41860,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>

</xml_diff>

<commit_message>
Simplify hybrid drainage to P-03/P-07/RP-02 topology
West surfaces share OUEST_P03_RP02; east trees to P-07 without CB
in strip; roof/tresfond via MEC to basin; readable Element_IDs.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
@@ -92,7 +92,7 @@
       <color rgb="001B4F72"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -166,6 +166,11 @@
         <fgColor rgb="00FCF3CF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -219,7 +224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -277,6 +282,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,551 +637,583 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="22" min="1" max="1"/>
-    <col width="12" customWidth="1" style="22" min="2" max="2"/>
+    <col width="28" customWidth="1" style="22" min="1" max="1"/>
+    <col width="16" customWidth="1" style="22" min="2" max="2"/>
     <col width="28" customWidth="1" style="22" min="3" max="3"/>
-    <col width="10" customWidth="1" style="22" min="4" max="4"/>
-    <col width="18" customWidth="1" style="22" min="5" max="5"/>
-    <col width="36" customWidth="1" style="22" min="6" max="6"/>
+    <col width="22" customWidth="1" style="22" min="4" max="4"/>
+    <col width="40" customWidth="1" style="22" min="5" max="5"/>
+    <col width="20" customWidth="1" style="22" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>LECTURE RAPIDE — réseau hybride (plan 1796-C-03)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1" s="22">
+          <t>LECTURE RAPIDE — drainage SIMPLIFIÉ (plan 1796-C-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1" s="22">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Calcul: Zones_tributaires (Q) → Elements_hybrides Element_ID (O = Q local via SUMIFS sur J; P = amont; Q = design) → Noeuds_stockage. Si O=0: Zones!J doit égaler exactement Elements!A.</t>
+          <t>Idée: (1) Ouest surfaces → CB P-03 → RP-02 → rue. (2) Est arbres sans CB → ruissellement → CB P-07 → RP-02. (3) Toit + tréfond → mécanique intérieur → bassin. Grass vs pavage = zones séparées (C différent), même conduite ouest.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
         <is>
-          <t>1) CHAÎNE EST</t>
+          <t>A) OUEST — comment gérer grass / pavage</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>Ordre</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>C (Inputs)</t>
+        </is>
+      </c>
+      <c r="D5" s="43" t="inlineStr">
+        <is>
+          <t>Où ça va</t>
+        </is>
+      </c>
+      <c r="E5" s="43" t="inlineStr">
+        <is>
+          <t>Pourquoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>Z04</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>Gazon</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="D6" s="44" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02 → P-03</t>
+        </is>
+      </c>
+      <c r="E6" s="44" t="inlineStr">
+        <is>
+          <t>Même CB, C plus faible</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="44" t="inlineStr">
+        <is>
+          <t>Z05</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>Gazon</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="D7" s="44" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02 → P-03</t>
+        </is>
+      </c>
+      <c r="E7" s="44" t="inlineStr">
+        <is>
+          <t>Idem</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>Z06</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>Gazon</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="D8" s="44" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02 → P-03</t>
+        </is>
+      </c>
+      <c r="E8" s="44" t="inlineStr">
+        <is>
+          <t>Idem</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>Z07</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>Pavé-uni</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02 → P-03</t>
+        </is>
+      </c>
+      <c r="E9" s="44" t="inlineStr">
+        <is>
+          <t>Même CB, C élevé</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>Z08</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>Pavé-uni</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="D10" s="44" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02 → P-03</t>
+        </is>
+      </c>
+      <c r="E10" s="44" t="inlineStr">
+        <is>
+          <t>Idem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>B) EST — bande arbres (jaune) sans CB + P-07 sud</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
         <is>
           <t>Element_ID</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
-        <is>
-          <t>Noeuds (plan)</t>
-        </is>
-      </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
+        <is>
+          <t>Noeuds</t>
+        </is>
+      </c>
+      <c r="E13" s="43" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>Z03</t>
+        </is>
+      </c>
+      <c r="B14" s="45" t="inlineStr">
+        <is>
+          <t>Arbres/gazon</t>
+        </is>
+      </c>
+      <c r="C14" s="45" t="inlineStr">
+        <is>
+          <t>EST_ARBRES_VERS_P07</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>BANDE_ARBRES → P-07</t>
+        </is>
+      </c>
+      <c r="E14" s="45" t="inlineStr">
+        <is>
+          <t>Pas de CB dans la bande (seulement arbres)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="45" t="inlineStr">
+        <is>
+          <t>Z10–Z12</t>
+        </is>
+      </c>
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>Sud-est</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="inlineStr">
+        <is>
+          <t>EST_P07_RP02</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>P-07 → RP-02</t>
+        </is>
+      </c>
+      <c r="E15" s="45" t="inlineStr">
+        <is>
+          <t>CB unique côté est: P-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>C) TOIT + TRÉFOND — mécanique → bassin</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Element_ID</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>Parcours</t>
+        </is>
+      </c>
+      <c r="E18" s="43" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>Z01</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>Toiture C≈0.95</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
+        </is>
+      </c>
+      <c r="D19" s="46" t="inlineStr">
+        <is>
+          <t>MEC-OUT → BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E19" s="46" t="inlineStr">
+        <is>
+          <t>Canalisé dans le bâtiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="46" t="inlineStr">
+        <is>
+          <t>Z02</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>Tréfond C≈0.95</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
+        </is>
+      </c>
+      <c r="D20" s="46" t="inlineStr">
+        <is>
+          <t>MEC-OUT → BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="inlineStr">
+        <is>
+          <t>Puisards / MEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>Z13</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>Strip nord</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
+        </is>
+      </c>
+      <c r="D21" s="46" t="inlineStr">
+        <is>
+          <t>MEC-OUT → BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>Vers mécanique</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>D) Éléments (noms lisibles — plus de E05C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>Element_ID</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
-        <is>
-          <t>Zones</t>
-        </is>
-      </c>
-      <c r="F5" s="31" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B6" s="32" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="C6" s="32" t="inlineStr">
-        <is>
-          <t>P-01 → P-02</t>
-        </is>
-      </c>
-      <c r="D6" s="32" t="inlineStr">
-        <is>
-          <t>TRENCH</t>
-        </is>
-      </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>De → Vers</t>
+        </is>
+      </c>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>Reçoit amont</t>
+        </is>
+      </c>
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>Rôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="42" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="C25" s="42" t="inlineStr">
+        <is>
+          <t>P-03 → RP-02</t>
+        </is>
+      </c>
+      <c r="D25" s="42" t="inlineStr">
+        <is>
+          <t>zones ouest</t>
+        </is>
+      </c>
+      <c r="E25" s="42" t="inlineStr">
+        <is>
+          <t>Collecte ouest</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="42" t="inlineStr">
+        <is>
+          <t>EST_ARBRES_VERS_P07</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>SWALE</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="inlineStr">
+        <is>
+          <t>BANDE_ARBRES → P-07</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
         <is>
           <t>Z03</t>
         </is>
       </c>
-      <c r="F6" s="32" t="inlineStr">
-        <is>
-          <t>Tranchée amont</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="32" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>E02</t>
-        </is>
-      </c>
-      <c r="C7" s="32" t="inlineStr">
-        <is>
-          <t>P-02 → P-03</t>
-        </is>
-      </c>
-      <c r="D7" s="32" t="inlineStr">
-        <is>
-          <t>TRENCH</t>
-        </is>
-      </c>
-      <c r="E7" s="32" t="inlineStr">
-        <is>
-          <t>(transfert)</t>
-        </is>
-      </c>
-      <c r="F7" s="32" t="inlineStr">
-        <is>
-          <t>Tranchée aval</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="32" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="32" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="C8" s="32" t="inlineStr">
-        <is>
-          <t>P-03 → MH-BASSIN-EST</t>
-        </is>
-      </c>
-      <c r="D8" s="32" t="inlineStr">
+      <c r="E26" s="42" t="inlineStr">
+        <is>
+          <t>Sans CB dans bande</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>EST_P07_RP02</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="E8" s="32" t="inlineStr">
-        <is>
-          <t>Z10,Z11,Z12</t>
-        </is>
-      </c>
-      <c r="F8" s="32" t="inlineStr">
-        <is>
-          <t>Entrée est</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="32" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>E07</t>
-        </is>
-      </c>
-      <c r="C9" s="32" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-EST → BASSIN-RET</t>
-        </is>
-      </c>
-      <c r="D9" s="32" t="inlineStr">
+      <c r="C27" s="42" t="inlineStr">
+        <is>
+          <t>P-07 → RP-02</t>
+        </is>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>arbres + sud-est</t>
+        </is>
+      </c>
+      <c r="E27" s="42" t="inlineStr">
+        <is>
+          <t>CB est</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="E9" s="32" t="inlineStr">
-        <is>
-          <t>(transfert)</t>
-        </is>
-      </c>
-      <c r="F9" s="32" t="inlineStr">
-        <is>
-          <t>BR.PLU est</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>2) CHAÎNE OUEST</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="31" t="inlineStr">
-        <is>
-          <t>Ordre</t>
-        </is>
-      </c>
-      <c r="B12" s="31" t="inlineStr">
-        <is>
-          <t>Element_ID</t>
-        </is>
-      </c>
-      <c r="C12" s="31" t="inlineStr">
-        <is>
-          <t>Noeuds</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E12" s="31" t="inlineStr">
-        <is>
-          <t>Zones</t>
-        </is>
-      </c>
-      <c r="F12" s="31" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B13" s="32" t="inlineStr">
-        <is>
-          <t>E05A</t>
-        </is>
-      </c>
-      <c r="C13" s="32" t="inlineStr">
-        <is>
-          <t>P-W1 → P-W2</t>
-        </is>
-      </c>
-      <c r="D13" s="32" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
+        <is>
+          <t>MEC-OUT → BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>Z01,Z02,Z13</t>
+        </is>
+      </c>
+      <c r="E28" s="42" t="inlineStr">
+        <is>
+          <t>Mécanique</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>RP02_VERS_RUE</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="E13" s="32" t="inlineStr">
-        <is>
-          <t>Z04</t>
-        </is>
-      </c>
-      <c r="F13" s="32" t="inlineStr">
-        <is>
-          <t>Gazon amont</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="32" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B14" s="32" t="inlineStr">
-        <is>
-          <t>E05B</t>
-        </is>
-      </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>P-W2 → P-W3</t>
-        </is>
-      </c>
-      <c r="D14" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E14" s="32" t="inlineStr">
-        <is>
-          <t>Z07</t>
-        </is>
-      </c>
-      <c r="F14" s="32" t="inlineStr">
-        <is>
-          <t>Pavé-uni</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="32" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>E05C</t>
-        </is>
-      </c>
-      <c r="C15" s="32" t="inlineStr">
-        <is>
-          <t>P-W3 → P-W4</t>
-        </is>
-      </c>
-      <c r="D15" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E15" s="32" t="inlineStr">
-        <is>
-          <t>Z05</t>
-        </is>
-      </c>
-      <c r="F15" s="32" t="inlineStr">
-        <is>
-          <t>Gazon milieu</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="32" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B16" s="32" t="inlineStr">
-        <is>
-          <t>E05D</t>
-        </is>
-      </c>
-      <c r="C16" s="32" t="inlineStr">
-        <is>
-          <t>P-W4 → P-W5</t>
-        </is>
-      </c>
-      <c r="D16" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E16" s="32" t="inlineStr">
-        <is>
-          <t>Z08</t>
-        </is>
-      </c>
-      <c r="F16" s="32" t="inlineStr">
-        <is>
-          <t>Pavé principal</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="32" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B17" s="32" t="inlineStr">
-        <is>
-          <t>E05E</t>
-        </is>
-      </c>
-      <c r="C17" s="32" t="inlineStr">
-        <is>
-          <t>P-W5 → P-W6</t>
-        </is>
-      </c>
-      <c r="D17" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E17" s="32" t="inlineStr">
-        <is>
-          <t>Z06</t>
-        </is>
-      </c>
-      <c r="F17" s="32" t="inlineStr">
-        <is>
-          <t>Gazon aval</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="32" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B18" s="32" t="inlineStr">
-        <is>
-          <t>E04</t>
-        </is>
-      </c>
-      <c r="C18" s="32" t="inlineStr">
-        <is>
-          <t>P-W6 → MH-BASSIN-OUEST</t>
-        </is>
-      </c>
-      <c r="D18" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E18" s="32" t="inlineStr">
-        <is>
-          <t>(transfert)</t>
-        </is>
-      </c>
-      <c r="F18" s="32" t="inlineStr">
-        <is>
-          <t>Lien coin</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B19" s="32" t="inlineStr">
-        <is>
-          <t>E08</t>
-        </is>
-      </c>
-      <c r="C19" s="32" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST → RP-02</t>
-        </is>
-      </c>
-      <c r="D19" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E19" s="32" t="inlineStr">
-        <is>
-          <t>(transfert)</t>
-        </is>
-      </c>
-      <c r="F19" s="32" t="inlineStr">
-        <is>
-          <t>Exutoire Ø300</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="30" t="inlineStr">
-        <is>
-          <t>3) MÉCANIQUE / TOITURE (P-011, P-08, P-09, CAN-010)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="31" t="inlineStr">
-        <is>
-          <t>Ordre</t>
-        </is>
-      </c>
-      <c r="B23" s="31" t="inlineStr">
-        <is>
-          <t>Element_ID</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>Noeuds</t>
-        </is>
-      </c>
-      <c r="D23" s="31" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E23" s="31" t="inlineStr">
-        <is>
-          <t>Zones</t>
-        </is>
-      </c>
-      <c r="F23" s="31" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t>E09</t>
-        </is>
-      </c>
-      <c r="C24" s="32" t="inlineStr">
-        <is>
-          <t>P-011 → BASSIN-RET</t>
-        </is>
-      </c>
-      <c r="D24" s="32" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="E24" s="32" t="inlineStr">
-        <is>
-          <t>Z01,Z02,Z13</t>
-        </is>
-      </c>
-      <c r="F24" s="32" t="inlineStr">
-        <is>
-          <t>Toit+tréfond+strip</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="33" t="inlineStr">
-        <is>
-          <t>4) BASSIN-RET = stockage (reçoit E07+E08+E09). Ne pas y router les zones pour le calcul O des conduites.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="34" t="inlineStr">
-        <is>
-          <t>Plan sud P-04 / P-05 / P-06 : présents sur PDF; à rattacher finement à la chaîne exutoire si vous scindez E08 plus tard.</t>
+      <c r="C29" s="42" t="inlineStr">
+        <is>
+          <t>RP-02 → RS-EX</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>ouest + est</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>Sortie rue</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="34" t="inlineStr">
+        <is>
+          <t>Longueurs P-03→RP-02 (2.3 m) et P-07→RP-02 (8.8 m) = démarrage selon cotations plan; ajuster dans Elements col F si votre métrique diffère.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1753,28 +1808,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1) Bande est (arbres): tranchee drainante + underdrain (E01/E02) au lieu d une noue profonde.</t>
+          <t>1) Est: bande arbres SANS CB → ruissellement vers P-07; pipe P-07→RP-02.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2) Bande sud (2.0 m): noue lineaire + volume de retention dans le corridor contraint.</t>
+          <t>2) Ouest: surfaces grass/pavage → CB P-03 → RP-02 → rue.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3) Ouest: drainage en conduites (DN250/DN300) vers E04 puis entree ouest bassin.</t>
+          <t>3) Toit + tréfond: mécanique intérieur → bassin de rétention.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4) Zone grise est (tresfond): puisards + reseau interne mecanique vers sortie sud et bassin.</t>
+          <t>4) Noms lisibles: OUEST_P03_RP02, EST_ARBRES_VERS_P07, EST_P07_RP02, MEC_TOIT_TRESFOND_BASSIN, RP02_VERS_RUE.</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1880,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>East strip total width (m)</t>
+          <t>East trees strip (no CB)</t>
         </is>
       </c>
       <c r="B11" s="5">
@@ -1834,12 +1889,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>&lt;= site 2.5 m</t>
+          <t>Bande arbres (pas de CB)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>EST_ARBRES_VERS_P07</t>
         </is>
       </c>
       <c r="F11" s="3">
@@ -1858,7 +1913,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Underdrain trench width x depth (m)</t>
+          <t>East CB P-07 pipe</t>
         </is>
       </c>
       <c r="B12" s="5">
@@ -1867,12 +1922,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Tree-compatible trench</t>
+          <t>CB P-07 sud → RP-02</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="F12" s="3">
@@ -1891,7 +1946,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Underdrain diameter (mm)</t>
+          <t>West CB P-03 pipe</t>
         </is>
       </c>
       <c r="B13" s="5">
@@ -1900,12 +1955,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Initial recommendation</t>
+          <t>CB P-03 ouest → RP-02</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="F13" s="3">
@@ -1924,7 +1979,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>West connector to basin inlet (m)</t>
+          <t>Outlet to street</t>
         </is>
       </c>
       <c r="B14" s="5">
@@ -1933,13 +1988,13 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Measured corner link P-W6 -&gt; MH-BASSIN-OUEST</t>
+          <t>RP-02 → réseau existant</t>
         </is>
       </c>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>RP02_VERS_RUE</t>
         </is>
       </c>
       <c r="F14" s="3">
@@ -1967,14 +2022,14 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Storage geometry at node BASSIN-RET (not an E04 reach).</t>
+          <t>Storage at BASSIN-RET (toit/tréfond via MEC)</t>
         </is>
       </c>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>BASSIN-RET (node)</t>
+          <t>BASSIN-RET</t>
         </is>
       </c>
       <c r="G15" s="16" t="n"/>
@@ -1991,18 +2046,18 @@
         </is>
       </c>
       <c r="B16" s="10">
-        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E07",Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("MEC_TOIT_TRESFOND_BASSIN",Elements_hybrides!$A$4:$A$204,0)),"")</f>
         <v/>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>MH-BASSIN-EST -&gt; BASSIN-RET</t>
+          <t>MEC-OUT → BASSIN-RET</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="F16" s="3">
@@ -2025,18 +2080,18 @@
         </is>
       </c>
       <c r="B17" s="16">
-        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("E08",Elements_hybrides!$A$4:$A$204,0)),"")</f>
+        <f>IFERROR(INDEX(Elements_hybrides!$F$4:$F$204,MATCH("RP02_VERS_RUE",Elements_hybrides!$A$4:$A$204,0)),"")</f>
         <v/>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>MH-BASSIN-OUEST -&gt; RP-02 / bassin path</t>
+          <t>RP-02 → RS-EX</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>RP02_VERS_RUE</t>
         </is>
       </c>
       <c r="F17" s="3">
@@ -2270,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="145" customWidth="1" style="22" min="1" max="1"/>
@@ -2673,6 +2728,34 @@
       <c r="A61" t="inlineStr">
         <is>
           <t>- Voir onglets Lecture_rapide et Convention_labels. Elements AM:AM = libellé plan / zones liées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="35" t="inlineStr">
+        <is>
+          <t>SIMPLIFICATION majeure (demande utilisateur):</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>- Ouest: un seul CB P-03 → RP-02 (plus de chaîne E05A…E05E). Grass/pavage = zones séparées, même Element_ID OUEST_P03_RP02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>- Est: bande arbres sans CB → EST_ARBRES_VERS_P07; CB P-07 sud → RP-02.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>- Toit+tréfond: MEC_TOIT_TRESFOND_BASSIN vers bassin. Voir Lecture_rapide.</t>
         </is>
       </c>
     </row>
@@ -3976,9 +4059,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="K2" s="36" t="inlineStr">
-        <is>
-          <t>CRITIQUE: J = Element_ID de Elements_hybrides!A (E01, E05A…). Pas un Node_ID (P-01, RP-02) ni BASSIN-RET pour toiture.</t>
+      <c r="K2" s="47" t="inlineStr">
+        <is>
+          <t>Surfaces différentes (grass C=0.25, pavage/toit C=0.95): une zone par type, mais plusieurs zones peuvent partager le même Element_ID (ex. tout l'ouest → OUEST_P03_RP02). J doit égaler exactement Elements!A.</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4145,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Toiture principale (bloc jaune)</t>
+          <t>TOITURE — via drainage mécanique intérieur → bassin</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4092,12 +4175,12 @@
       </c>
       <c r="J4" s="37" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Toiture → mécanique P-011 (plan) → E09 → bassin. PAS BASSIN-RET (sinon O=0 sur conduites).</t>
+          <t>Route → MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="L4" s="4" t="n">
@@ -4120,7 +4203,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tresfond est (gris)</t>
+          <t>TRÉFOND (gris) — puisards/MEC intérieur → bassin</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -4150,12 +4233,12 @@
       </c>
       <c r="J5" s="37" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Tréfond gris est → puisards MEC → P-011 → E09.</t>
+          <t>Route → MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="L5" s="4" t="n">
@@ -4178,7 +4261,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Bande verte est (arbres)</t>
+          <t>EST ARBRES (bande jaune) — pas de CB dans la bande; ruissellement vers P-07</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -4208,12 +4291,12 @@
       </c>
       <c r="J6" s="37" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>EST_ARBRES_VERS_P07</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Bande verte est → tranchée E01 (P-01→P-02).</t>
+          <t>Route → EST_ARBRES_VERS_P07</t>
         </is>
       </c>
       <c r="L6" s="4" t="n">
@@ -4236,7 +4319,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon amont (12.5 m2)</t>
+          <t>OUEST gazon amont — vers CB P-03</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -4266,12 +4349,12 @@
       </c>
       <c r="J7" s="37" t="inlineStr">
         <is>
-          <t>E05A</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon amont → E05A (P-W1→P-W2).</t>
+          <t>Route → OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="L7" s="4" t="n">
@@ -4294,7 +4377,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ouest pave-uni court (6.7 m2)</t>
+          <t>OUEST pavé-uni court — vers CB P-03</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -4324,12 +4407,12 @@
       </c>
       <c r="J8" s="37" t="inlineStr">
         <is>
-          <t>E05B</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Ouest pavé-uni → E05B.</t>
+          <t>Route → OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="L8" s="4" t="n">
@@ -4352,7 +4435,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon milieu (27.2 m2)</t>
+          <t>OUEST gazon milieu — vers CB P-03</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -4382,12 +4465,12 @@
       </c>
       <c r="J9" s="37" t="inlineStr">
         <is>
-          <t>E05C</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon milieu → E05C.</t>
+          <t>Route → OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="L9" s="4" t="n">
@@ -4410,7 +4493,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Ouest pave-uni principal (37.5 m2)</t>
+          <t>OUEST pavé-uni principal — vers CB P-03</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -4440,12 +4523,12 @@
       </c>
       <c r="J10" s="37" t="inlineStr">
         <is>
-          <t>E05D</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Ouest pavé-uni principal → E05D.</t>
+          <t>Route → OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="L10" s="4" t="n">
@@ -4468,7 +4551,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon aval coin sud-ouest (21.9 m2)</t>
+          <t>OUEST gazon aval — vers CB P-03</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -4498,12 +4581,12 @@
       </c>
       <c r="J11" s="37" t="inlineStr">
         <is>
-          <t>E05E</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Ouest gazon aval → E05E.</t>
+          <t>Route → OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="L11" s="4" t="n">
@@ -4526,7 +4609,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Empreinte bassin retention (zone de stockage)</t>
+          <t>Empreinte bassin — non contributive</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -4555,7 +4638,7 @@
       <c r="J12" s="38" t="n"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Empreinte bassin — non contributive (Inputs!B52).</t>
+          <t>Non contributive</t>
         </is>
       </c>
       <c r="L12" s="4" t="n">
@@ -4578,7 +4661,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Sud gris local (pavage)</t>
+          <t>SUD-EST pavage — vers CB P-07</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -4608,12 +4691,12 @@
       </c>
       <c r="J13" s="37" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Sud/est pavage → E03.</t>
+          <t>Route → EST_P07_RP02</t>
         </is>
       </c>
       <c r="L13" s="4" t="n">
@@ -4636,7 +4719,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sud est vert</t>
+          <t>SUD-EST gazon — vers CB P-07</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -4666,12 +4749,12 @@
       </c>
       <c r="J14" s="37" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Sud est vert → E03.</t>
+          <t>Route → EST_P07_RP02</t>
         </is>
       </c>
       <c r="L14" s="4" t="n">
@@ -4694,7 +4777,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Sud est gris petit (pavage)</t>
+          <t>SUD-EST pavage petit — vers CB P-07</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -4724,12 +4807,12 @@
       </c>
       <c r="J15" s="37" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Sud est pavage petit → E03.</t>
+          <t>Route → EST_P07_RP02</t>
         </is>
       </c>
       <c r="L15" s="4" t="n">
@@ -4752,7 +4835,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Petit strip vert nord (vers puisard PEHD central)</t>
+          <t>Strip nord — vers mécanique / bassin</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -4782,12 +4865,12 @@
       </c>
       <c r="J16" s="37" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Strip vert nord → mécanique → E09.</t>
+          <t>Route → MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="L16" s="4" t="n"/>
@@ -11267,9 +11350,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
-        <is>
-          <t>Legend: PIPE=blue, SWALE=green, TRENCH=orange, CHECK=red; AH connection status and AL drop check use Inputs!B54:B56 thresholds.</t>
+      <c r="A2" s="48" t="inlineStr">
+        <is>
+          <t>SIMPLIFIÉ selon plan 1796-C-03: Ouest→P-03→RP-02; Est arbres→P-07→RP-02; Toit/tréfond→mécanique→bassin. Element_ID lisibles (plus de E05C). Surfaces grass/pavage: zones séparées (C différent) mais même Element_ID ouest.</t>
         </is>
       </c>
     </row>
@@ -11481,61 +11564,50 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>TRENCH</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>P-01</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>P-02</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>E02</t>
+      <c r="A4" s="49" t="inlineStr">
+        <is>
+          <t>OUEST_P03_RP02</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="D4" s="49" t="inlineStr">
+        <is>
+          <t>RP-02</t>
+        </is>
+      </c>
+      <c r="E4" s="49" t="inlineStr">
+        <is>
+          <t>RP02_VERS_RUE</t>
         </is>
       </c>
       <c r="F4" s="8" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="G4" s="8">
-        <f>Inputs!$B$33</f>
-        <v/>
+        <v>2.3</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>0.022</v>
       </c>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="10">
         <f>IF(A4="","",IF(H4&lt;&gt;"",H4,IF(UPPER(TRIM(B4))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B4))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J4" s="8">
-        <f>Inputs!$B$30</f>
-        <v/>
-      </c>
-      <c r="K4" s="8">
-        <f>Inputs!$B$28</f>
-        <v/>
-      </c>
-      <c r="L4" s="8">
-        <f>Inputs!$B$29</f>
-        <v/>
-      </c>
-      <c r="M4" s="8" t="n">
+      <c r="J4" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="K4" s="8" t="n"/>
+      <c r="L4" s="8" t="n"/>
+      <c r="M4" s="8" t="n"/>
+      <c r="N4" s="8" t="n">
         <v>0</v>
-      </c>
-      <c r="N4" s="8">
-        <f>Inputs!$B$22</f>
-        <v/>
       </c>
       <c r="O4" s="10">
         <f>IF(A4="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A4))</f>
@@ -11591,7 +11663,7 @@
       </c>
       <c r="AB4" s="3" t="inlineStr">
         <is>
-          <t>Longueur corrigee selon plan: P-01 -&gt; P-02 = 9.6 m.</t>
+          <t>CB ouest P-03 (gazon+pavé) → regard RP-02. Surfaces distinctes restent en Zones (C différent), même Element_ID.</t>
         </is>
       </c>
       <c r="AC4" s="8" t="n"/>
@@ -11633,7 +11705,7 @@
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>Tranchée est P-01→P-02 (bande arbres)</t>
+          <t>Plan: P-03 → RP-02</t>
         </is>
       </c>
       <c r="AN4" s="39">
@@ -11642,66 +11714,59 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>Z03</t>
+          <t>Z04,Z05,Z06,Z07,Z08</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>E02</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>TRENCH</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>P-02</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>P-03</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>E03</t>
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>EST_ARBRES_VERS_P07</t>
+        </is>
+      </c>
+      <c r="B5" s="37" t="inlineStr">
+        <is>
+          <t>SWALE</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>BANDE_ARBRES</t>
+        </is>
+      </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="E5" s="37" t="inlineStr">
+        <is>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="F5" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G5" s="8">
-        <f>Inputs!$B$33</f>
-        <v/>
+        <v>20</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>0.01</v>
       </c>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="10">
         <f>IF(A5="","",IF(H5&lt;&gt;"",H5,IF(UPPER(TRIM(B5))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B5))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J5" s="8">
-        <f>Inputs!$B$30</f>
-        <v/>
-      </c>
-      <c r="K5" s="8">
-        <f>Inputs!$B$28</f>
-        <v/>
-      </c>
-      <c r="L5" s="8">
-        <f>Inputs!$B$29</f>
-        <v/>
+      <c r="J5" s="8" t="n"/>
+      <c r="K5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>0.1</v>
       </c>
       <c r="M5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="8">
-        <f>Inputs!$B$22</f>
-        <v/>
+      <c r="N5" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O5" s="10">
         <f>IF(A5="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A5))</f>
@@ -11757,7 +11822,7 @@
       </c>
       <c r="AB5" s="3" t="inlineStr">
         <is>
-          <t>Longueur corrigee selon plan: P-02 -&gt; P-03 = 8.7 m.</t>
+          <t>Bande est jaune/arbres: PAS de CB dans la bande. Ruissellement de surface vers P-07 au sud. Modélisé SWALE/collecte.</t>
         </is>
       </c>
       <c r="AC5" s="8" t="n"/>
@@ -11799,7 +11864,7 @@
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>Tranchée est P-02→P-03</t>
+          <t>Plan: arbres (cercles) → P-07 sud</t>
         </is>
       </c>
       <c r="AN5" s="39">
@@ -11808,41 +11873,41 @@
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>(aucune — transfert amont)</t>
+          <t>Z03</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>EST_P07_RP02</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>P-03</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-EST</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>E07</t>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>RP-02</t>
+        </is>
+      </c>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>RP02_VERS_RUE</t>
         </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>16.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0025</v>
       </c>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="10">
@@ -11850,7 +11915,7 @@
         <v/>
       </c>
       <c r="J6" s="8" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="8" t="n"/>
@@ -11912,7 +11977,7 @@
       </c>
       <c r="AB6" s="3" t="inlineStr">
         <is>
-          <t>Entree EST: P-03 -&gt; MH-BASSIN-EST (16.1 m).</t>
+          <t>CB est P-07 (sud) → RP-02. Reçoit aussi pavage/gazon sud locaux.</t>
         </is>
       </c>
       <c r="AC6" s="8" t="n"/>
@@ -11954,7 +12019,7 @@
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>PIPE P-03→MH-BASSIN-EST</t>
+          <t>Plan: P-07 Ø300 L≈8.8 m</t>
         </is>
       </c>
       <c r="AN6" s="39">
@@ -11963,50 +12028,47 @@
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>Z10, Z11, Z12</t>
+          <t>Z10,Z11,Z12</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>E04</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>P-W6</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>E08</t>
-        </is>
-      </c>
+      <c r="C7" s="50" t="inlineStr">
+        <is>
+          <t>MEC-OUT</t>
+        </is>
+      </c>
+      <c r="D7" s="50" t="inlineStr">
+        <is>
+          <t>BASSIN-RET</t>
+        </is>
+      </c>
+      <c r="E7" s="50" t="n"/>
       <c r="F7" s="8">
-        <f>Inputs!$B$53</f>
+        <f>Inputs!$B$60</f>
         <v/>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="10">
         <f>IF(A7="","",IF(H7&lt;&gt;"",H7,IF(UPPER(TRIM(B7))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B7))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J7" s="8" t="n">
-        <v>250</v>
+      <c r="J7" s="8">
+        <f>Inputs!$B$61</f>
+        <v/>
       </c>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
@@ -12068,7 +12130,7 @@
       </c>
       <c r="AB7" s="3" t="inlineStr">
         <is>
-          <t>Collecteur ouest final en conduite (4.7 m) vers entree ouest bassin.</t>
+          <t>Toiture + tréfond + strip nord: drainage MÉCANIQUE intérieur → bassin sud.</t>
         </is>
       </c>
       <c r="AC7" s="8" t="n"/>
@@ -12110,7 +12172,7 @@
       </c>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>PIPE P-W6→MH-BASSIN-OUEST</t>
+          <t>Plan: VOIR MEC / P-011 / CAN-010 → bassin</t>
         </is>
       </c>
       <c r="AN7" s="39">
@@ -12119,42 +12181,37 @@
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>(aucune — transfert amont)</t>
+          <t>Z01,Z02,Z13</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>E05A</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>RP02_VERS_RUE</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
         <is>
           <t>PIPE</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>P-W1</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>P-W2</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>E05B</t>
-        </is>
-      </c>
-      <c r="F8" s="12">
-        <f>Inputs!$B$48</f>
-        <v/>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>RP-02</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>RS-EX</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="n"/>
+      <c r="F8" s="12" t="n">
+        <v>16.6</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="10">
@@ -12162,7 +12219,7 @@
         <v/>
       </c>
       <c r="J8" s="8" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="K8" s="8" t="n"/>
       <c r="L8" s="8" t="n"/>
@@ -12224,7 +12281,7 @@
       </c>
       <c r="AB8" s="3" t="inlineStr">
         <is>
-          <t>Ouest segment amont en conduite DN250 vers E05B.</t>
+          <t>Regard RP-02 vers raccordement réseau existant (rue). Reçoit OUEST_P03_RP02 + EST_P07_RP02.</t>
         </is>
       </c>
       <c r="AC8" s="8" t="n"/>
@@ -12266,7 +12323,7 @@
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>PIPE ouest P-W1→P-W2</t>
+          <t>Plan: RP-02 → existant (Ø300)</t>
         </is>
       </c>
       <c r="AN8" s="39">
@@ -12275,57 +12332,28 @@
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>Z04</t>
+          <t>(transfert amont)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>E05B</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>P-W2</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>P-W3</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>E05C</t>
-        </is>
-      </c>
-      <c r="F9" s="12">
-        <f>Inputs!$B$42</f>
-        <v/>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="10">
         <f>IF(A9="","",IF(H9&lt;&gt;"",H9,IF(UPPER(TRIM(B9))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B9))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J9" s="8" t="n">
-        <v>200</v>
-      </c>
+      <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
       <c r="M9" s="8" t="n"/>
-      <c r="N9" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N9" s="8" t="n"/>
       <c r="O9" s="10">
         <f>IF(A9="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A9))</f>
         <v/>
@@ -12378,11 +12406,7 @@
         <f>IF(A9="","",IF(OR(U9&gt;1,AND(X9&lt;&gt;"",X9&lt;Inputs!$B$16),AND(X9&lt;&gt;"",X9&gt;Inputs!$B$17),G9&lt;Inputs!$B$18,AH9="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB9" s="3" t="inlineStr">
-        <is>
-          <t>Traverse pave-uni court en conduite DN250 (strategy ouest tout-pipe).</t>
-        </is>
-      </c>
+      <c r="AB9" s="3" t="n"/>
       <c r="AC9" s="8" t="n"/>
       <c r="AD9" s="10">
         <f>IF(A9="","",IF(AC9&lt;&gt;"",AC9,IF(E9="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E9,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B9))="SWALE",UPPER(TRIM(AI9))="PIPE"),AND(UPPER(TRIM(B9))="TRENCH",UPPER(TRIM(AI9))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -12420,68 +12444,29 @@
         <f>IF(A9="","",IF(E9="","TERMINAL",IF(OR(AND(UPPER(TRIM(B9))="SWALE",UPPER(TRIM(AI9))="PIPE"),AND(UPPER(TRIM(B9))="TRENCH",UPPER(TRIM(AI9))="PIPE")),IF(OR(AG9="",AJ9="",AK9=""),"INFO",IF(AND(AG9&gt;=AJ9,AG9&lt;=AK9),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>PIPE ouest P-W2→P-W3</t>
-        </is>
-      </c>
       <c r="AN9" s="39">
         <f>IF(A9="","",COUNTIF(Zones_tributaires!$J:$J,A9))</f>
         <v/>
       </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>Z07</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>E05C</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>P-W3</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>P-W4</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>E05D</t>
-        </is>
-      </c>
-      <c r="F10" s="12">
-        <f>Inputs!$B$49</f>
-        <v/>
-      </c>
-      <c r="G10" s="8" t="n">
-        <v>0.008999999999999999</v>
-      </c>
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="10">
         <f>IF(A10="","",IF(H10&lt;&gt;"",H10,IF(UPPER(TRIM(B10))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B10))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J10" s="8" t="n">
-        <v>200</v>
-      </c>
+      <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="8" t="n"/>
       <c r="M10" s="8" t="n"/>
-      <c r="N10" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N10" s="8" t="n"/>
       <c r="O10" s="10">
         <f>IF(A10="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A10))</f>
         <v/>
@@ -12534,11 +12519,7 @@
         <f>IF(A10="","",IF(OR(U10&gt;1,AND(X10&lt;&gt;"",X10&lt;Inputs!$B$16),AND(X10&lt;&gt;"",X10&gt;Inputs!$B$17),G10&lt;Inputs!$B$18,AH10="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB10" s="3" t="inlineStr">
-        <is>
-          <t>Ouest segment milieu en conduite DN300 vers E05D.</t>
-        </is>
-      </c>
+      <c r="AB10" s="3" t="n"/>
       <c r="AC10" s="8" t="n"/>
       <c r="AD10" s="10">
         <f>IF(A10="","",IF(AC10&lt;&gt;"",AC10,IF(E10="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E10,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B10))="SWALE",UPPER(TRIM(AI10))="PIPE"),AND(UPPER(TRIM(B10))="TRENCH",UPPER(TRIM(AI10))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -12576,68 +12557,29 @@
         <f>IF(A10="","",IF(E10="","TERMINAL",IF(OR(AND(UPPER(TRIM(B10))="SWALE",UPPER(TRIM(AI10))="PIPE"),AND(UPPER(TRIM(B10))="TRENCH",UPPER(TRIM(AI10))="PIPE")),IF(OR(AG10="",AJ10="",AK10=""),"INFO",IF(AND(AG10&gt;=AJ10,AG10&lt;=AK10),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>PIPE ouest P-W3→P-W4</t>
-        </is>
-      </c>
       <c r="AN10" s="39">
         <f>IF(A10="","",COUNTIF(Zones_tributaires!$J:$J,A10))</f>
         <v/>
       </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>Z05</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>E05D</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>P-W4</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>P-W5</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>E05E</t>
-        </is>
-      </c>
-      <c r="F11" s="12">
-        <f>Inputs!$B$43</f>
-        <v/>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>0.008999999999999999</v>
-      </c>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="10">
         <f>IF(A11="","",IF(H11&lt;&gt;"",H11,IF(UPPER(TRIM(B11))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B11))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J11" s="8" t="n">
-        <v>200</v>
-      </c>
+      <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="8" t="n"/>
-      <c r="N11" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N11" s="8" t="n"/>
       <c r="O11" s="10">
         <f>IF(A11="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A11))</f>
         <v/>
@@ -12690,11 +12632,7 @@
         <f>IF(A11="","",IF(OR(U11&gt;1,AND(X11&lt;&gt;"",X11&lt;Inputs!$B$16),AND(X11&lt;&gt;"",X11&gt;Inputs!$B$17),G11&lt;Inputs!$B$18,AH11="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB11" s="3" t="inlineStr">
-        <is>
-          <t>Traverse pave-uni principal en conduite DN300.</t>
-        </is>
-      </c>
+      <c r="AB11" s="3" t="n"/>
       <c r="AC11" s="8" t="n"/>
       <c r="AD11" s="10">
         <f>IF(A11="","",IF(AC11&lt;&gt;"",AC11,IF(E11="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E11,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B11))="SWALE",UPPER(TRIM(AI11))="PIPE"),AND(UPPER(TRIM(B11))="TRENCH",UPPER(TRIM(AI11))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -12732,68 +12670,29 @@
         <f>IF(A11="","",IF(E11="","TERMINAL",IF(OR(AND(UPPER(TRIM(B11))="SWALE",UPPER(TRIM(AI11))="PIPE"),AND(UPPER(TRIM(B11))="TRENCH",UPPER(TRIM(AI11))="PIPE")),IF(OR(AG11="",AJ11="",AK11=""),"INFO",IF(AND(AG11&gt;=AJ11,AG11&lt;=AK11),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>PIPE ouest P-W4→P-W5</t>
-        </is>
-      </c>
       <c r="AN11" s="39">
         <f>IF(A11="","",COUNTIF(Zones_tributaires!$J:$J,A11))</f>
         <v/>
       </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>Z08</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>E05E</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>P-W5</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>P-W6</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>E04</t>
-        </is>
-      </c>
-      <c r="F12" s="12">
-        <f>Inputs!$B$50</f>
-        <v/>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>0.008</v>
-      </c>
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="10">
         <f>IF(A12="","",IF(H12&lt;&gt;"",H12,IF(UPPER(TRIM(B12))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B12))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>200</v>
-      </c>
+      <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
-      <c r="N12" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N12" s="8" t="n"/>
       <c r="O12" s="10">
         <f>IF(A12="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A12))</f>
         <v/>
@@ -12846,11 +12745,7 @@
         <f>IF(A12="","",IF(OR(U12&gt;1,AND(X12&lt;&gt;"",X12&lt;Inputs!$B$16),AND(X12&lt;&gt;"",X12&gt;Inputs!$B$17),G12&lt;Inputs!$B$18,AH12="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB12" s="3" t="inlineStr">
-        <is>
-          <t>Ouest segment aval en conduite DN300 vers E04.</t>
-        </is>
-      </c>
+      <c r="AB12" s="3" t="n"/>
       <c r="AC12" s="8" t="n"/>
       <c r="AD12" s="10">
         <f>IF(A12="","",IF(AC12&lt;&gt;"",AC12,IF(E12="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E12,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B12))="SWALE",UPPER(TRIM(AI12))="PIPE"),AND(UPPER(TRIM(B12))="TRENCH",UPPER(TRIM(AI12))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -12888,38 +12783,16 @@
         <f>IF(A12="","",IF(E12="","TERMINAL",IF(OR(AND(UPPER(TRIM(B12))="SWALE",UPPER(TRIM(AI12))="PIPE"),AND(UPPER(TRIM(B12))="TRENCH",UPPER(TRIM(AI12))="PIPE")),IF(OR(AG12="",AJ12="",AK12=""),"INFO",IF(AND(AG12&gt;=AJ12,AG12&lt;=AK12),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>PIPE ouest P-W5→P-W6</t>
-        </is>
-      </c>
       <c r="AN12" s="39">
         <f>IF(A12="","",COUNTIF(Zones_tributaires!$J:$J,A12))</f>
         <v/>
       </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>Z06</t>
-        </is>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST</t>
-        </is>
-      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
@@ -13023,63 +12896,29 @@
         <f>IF(A13="","",IF(E13="","TERMINAL",IF(OR(AND(UPPER(TRIM(B13))="SWALE",UPPER(TRIM(AI13))="PIPE"),AND(UPPER(TRIM(B13))="TRENCH",UPPER(TRIM(AI13))="PIPE")),IF(OR(AG13="",AJ13="",AK13=""),"INFO",IF(AND(AG13&gt;=AJ13,AG13&lt;=AK13),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM13" t="inlineStr">
-        <is>
-          <t>Bassin EZ-STORM plan 2.44×34.4×1.22</t>
-        </is>
-      </c>
       <c r="AN13" s="39">
         <f>IF(A13="","",COUNTIF(Zones_tributaires!$J:$J,A13))</f>
         <v/>
       </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>(aucune — transfert amont)</t>
-        </is>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>E07</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-EST</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
-      <c r="F14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>0.005</v>
-      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="10">
         <f>IF(A14="","",IF(H14&lt;&gt;"",H14,IF(UPPER(TRIM(B14))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B14))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J14" s="8" t="n">
-        <v>300</v>
-      </c>
+      <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N14" s="8" t="n"/>
       <c r="O14" s="10">
         <f>IF(A14="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A14))</f>
         <v/>
@@ -13132,11 +12971,7 @@
         <f>IF(A14="","",IF(OR(U14&gt;1,AND(X14&lt;&gt;"",X14&lt;Inputs!$B$16),AND(X14&lt;&gt;"",X14&gt;Inputs!$B$17),G14&lt;Inputs!$B$18,AH14="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB14" s="3" t="inlineStr">
-        <is>
-          <t>Courte liaison d'entree/ouvrage de regulation vers noeud de stockage BASSIN-RET.</t>
-        </is>
-      </c>
+      <c r="AB14" s="3" t="n"/>
       <c r="AC14" s="8" t="n"/>
       <c r="AD14" s="10">
         <f>IF(A14="","",IF(AC14&lt;&gt;"",AC14,IF(E14="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E14,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B14))="SWALE",UPPER(TRIM(AI14))="PIPE"),AND(UPPER(TRIM(B14))="TRENCH",UPPER(TRIM(AI14))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -13174,63 +13009,29 @@
         <f>IF(A14="","",IF(E14="","TERMINAL",IF(OR(AND(UPPER(TRIM(B14))="SWALE",UPPER(TRIM(AI14))="PIPE"),AND(UPPER(TRIM(B14))="TRENCH",UPPER(TRIM(AI14))="PIPE")),IF(OR(AG14="",AJ14="",AK14=""),"INFO",IF(AND(AG14&gt;=AJ14,AG14&lt;=AK14),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM14" t="inlineStr">
-        <is>
-          <t>BR.PLU entrée est → BASSIN-RET</t>
-        </is>
-      </c>
       <c r="AN14" s="39">
         <f>IF(A14="","",COUNTIF(Zones_tributaires!$J:$J,A14))</f>
         <v/>
       </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>(aucune — transfert amont)</t>
-        </is>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>E08</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST</t>
-        </is>
-      </c>
-      <c r="D15" s="26" t="inlineStr">
-        <is>
-          <t>RP-02</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
-      <c r="F15" s="25" t="n">
-        <v>16.49</v>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>0.005</v>
-      </c>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="10">
         <f>IF(A15="","",IF(H15&lt;&gt;"",H15,IF(UPPER(TRIM(B15))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B15))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J15" s="8" t="n">
-        <v>300</v>
-      </c>
+      <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
-      <c r="N15" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N15" s="8" t="n"/>
       <c r="O15" s="10">
         <f>IF(A15="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A15))</f>
         <v/>
@@ -13283,11 +13084,7 @@
         <f>IF(A15="","",IF(OR(U15&gt;1,AND(X15&lt;&gt;"",X15&lt;Inputs!$B$16),AND(X15&lt;&gt;"",X15&gt;Inputs!$B$17),G15&lt;Inputs!$B$18,AH15="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB15" s="3" t="inlineStr">
-        <is>
-          <t>Entree OUEST: liaison caniveau/ouvrage vers bassin (2e entree).</t>
-        </is>
-      </c>
+      <c r="AB15" s="3" t="n"/>
       <c r="AC15" s="8" t="n"/>
       <c r="AD15" s="10">
         <f>IF(A15="","",IF(AC15&lt;&gt;"",AC15,IF(E15="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E15,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B15))="SWALE",UPPER(TRIM(AI15))="PIPE"),AND(UPPER(TRIM(B15))="TRENCH",UPPER(TRIM(AI15))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -13325,65 +13122,29 @@
         <f>IF(A15="","",IF(E15="","TERMINAL",IF(OR(AND(UPPER(TRIM(B15))="SWALE",UPPER(TRIM(AI15))="PIPE"),AND(UPPER(TRIM(B15))="TRENCH",UPPER(TRIM(AI15))="PIPE")),IF(OR(AG15="",AJ15="",AK15=""),"INFO",IF(AND(AG15&gt;=AJ15,AG15&lt;=AK15),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM15" t="inlineStr">
-        <is>
-          <t>Exutoire → RP-02 (≈L=16.6 m Ø300 plan)</t>
-        </is>
-      </c>
       <c r="AN15" s="39">
         <f>IF(A15="","",COUNTIF(Zones_tributaires!$J:$J,A15))</f>
         <v/>
       </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>(aucune — transfert amont)</t>
-        </is>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>E09</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>P-011</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
-      <c r="F16" s="8">
-        <f>Inputs!$B$60</f>
-        <v/>
-      </c>
-      <c r="G16" s="8" t="n">
-        <v>0.005</v>
-      </c>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="10">
         <f>IF(A16="","",IF(H16&lt;&gt;"",H16,IF(UPPER(TRIM(B16))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B16))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
         <v/>
       </c>
-      <c r="J16" s="8">
-        <f>Inputs!$B$61</f>
-        <v/>
-      </c>
+      <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n">
-        <v>0</v>
-      </c>
+      <c r="N16" s="8" t="n"/>
       <c r="O16" s="10">
         <f>IF(A16="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A16))</f>
         <v/>
@@ -13436,11 +13197,7 @@
         <f>IF(A16="","",IF(OR(U16&gt;1,AND(X16&lt;&gt;"",X16&lt;Inputs!$B$16),AND(X16&lt;&gt;"",X16&gt;Inputs!$B$17),G16&lt;Inputs!$B$18,AH16="CHECK"),"CHECK","OK"))</f>
         <v/>
       </c>
-      <c r="AB16" s="3" t="inlineStr">
-        <is>
-          <t>Apport puisards zone grise est via reseau interne mecanique (traversant batiment) vers bassin sud.</t>
-        </is>
-      </c>
+      <c r="AB16" s="3" t="n"/>
       <c r="AC16" s="8" t="n"/>
       <c r="AD16" s="10">
         <f>IF(A16="","",IF(AC16&lt;&gt;"",AC16,IF(E16="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E16,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B16))="SWALE",UPPER(TRIM(AI16))="PIPE"),AND(UPPER(TRIM(B16))="TRENCH",UPPER(TRIM(AI16))="PIPE")),Inputs!$B$57,0),""))))</f>
@@ -13478,19 +13235,9 @@
         <f>IF(A16="","",IF(E16="","TERMINAL",IF(OR(AND(UPPER(TRIM(B16))="SWALE",UPPER(TRIM(AI16))="PIPE"),AND(UPPER(TRIM(B16))="TRENCH",UPPER(TRIM(AI16))="PIPE")),IF(OR(AG16="",AJ16="",AK16=""),"INFO",IF(AND(AG16&gt;=AJ16,AG16&lt;=AK16),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
-      <c r="AM16" t="inlineStr">
-        <is>
-          <t>Mécanique P-011→BASSIN-RET</t>
-        </is>
-      </c>
       <c r="AN16" s="39">
         <f>IF(A16="","",COUNTIF(Zones_tributaires!$J:$J,A16))</f>
         <v/>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>Z01, Z02, Z13</t>
-        </is>
       </c>
     </row>
     <row r="17">
@@ -13601,6 +13348,10 @@
         <f>IF(A17="","",IF(E17="","TERMINAL",IF(OR(AND(UPPER(TRIM(B17))="SWALE",UPPER(TRIM(AI17))="PIPE"),AND(UPPER(TRIM(B17))="TRENCH",UPPER(TRIM(AI17))="PIPE")),IF(OR(AG17="",AJ17="",AK17=""),"INFO",IF(AND(AG17&gt;=AJ17,AG17&lt;=AK17),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
+      <c r="AN17">
+        <f>IF(A17="","",COUNTIF(Zones_tributaires!$J:$J,A17))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -13710,6 +13461,10 @@
         <f>IF(A18="","",IF(E18="","TERMINAL",IF(OR(AND(UPPER(TRIM(B18))="SWALE",UPPER(TRIM(AI18))="PIPE"),AND(UPPER(TRIM(B18))="TRENCH",UPPER(TRIM(AI18))="PIPE")),IF(OR(AG18="",AJ18="",AK18=""),"INFO",IF(AND(AG18&gt;=AJ18,AG18&lt;=AK18),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
+      <c r="AN18">
+        <f>IF(A18="","",COUNTIF(Zones_tributaires!$J:$J,A18))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -13819,6 +13574,10 @@
         <f>IF(A19="","",IF(E19="","TERMINAL",IF(OR(AND(UPPER(TRIM(B19))="SWALE",UPPER(TRIM(AI19))="PIPE"),AND(UPPER(TRIM(B19))="TRENCH",UPPER(TRIM(AI19))="PIPE")),IF(OR(AG19="",AJ19="",AK19=""),"INFO",IF(AND(AG19&gt;=AJ19,AG19&lt;=AK19),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
+      <c r="AN19">
+        <f>IF(A19="","",COUNTIF(Zones_tributaires!$J:$J,A19))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -13928,6 +13687,10 @@
         <f>IF(A20="","",IF(E20="","TERMINAL",IF(OR(AND(UPPER(TRIM(B20))="SWALE",UPPER(TRIM(AI20))="PIPE"),AND(UPPER(TRIM(B20))="TRENCH",UPPER(TRIM(AI20))="PIPE")),IF(OR(AG20="",AJ20="",AK20=""),"INFO",IF(AND(AG20&gt;=AJ20,AG20&lt;=AK20),"OK","CHECK")),"N/A")))</f>
         <v/>
       </c>
+      <c r="AN20">
+        <f>IF(A20="","",COUNTIF(Zones_tributaires!$J:$J,A20))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -13938,107 +13701,36 @@
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
-      <c r="I21" s="10">
-        <f>IF(A21="","",IF(H21&lt;&gt;"",H21,IF(UPPER(TRIM(B21))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B21))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
-        <v/>
-      </c>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
-      <c r="N21" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="10">
-        <f>IF(A21="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A21))</f>
-        <v/>
-      </c>
-      <c r="P21" s="10">
-        <f>IF(A21="","",SUMIFS($Q$4:$Q$204,$E$4:$E$204,$A21))</f>
-        <v/>
-      </c>
-      <c r="Q21" s="10">
-        <f>IF(A21="","",(O21+P21)*Inputs!$B$6)</f>
-        <v/>
-      </c>
-      <c r="R21" s="10">
-        <f>IF(A21="","",IF(UPPER(TRIM(B21))="PIPE",PI()*(J21/1000)^2/4,IF(OR(K21="",L21=""),"",L21*(K21+M21*L21))))</f>
-        <v/>
-      </c>
-      <c r="S21" s="10">
-        <f>IF(A21="","",IF(UPPER(TRIM(B21))="PIPE",(J21/1000)/4,IF(OR(R21="",K21="",L21=""),"",R21/(K21+2*L21*SQRT(1+M21^2)))))</f>
-        <v/>
-      </c>
-      <c r="T21" s="10">
-        <f>IF(A21="","",IF(OR(I21="",R21="",S21="",G21=""),"",(1/I21)*R21*(S21^(2/3))*SQRT(G21)))</f>
-        <v/>
-      </c>
-      <c r="U21" s="10">
-        <f>IF(OR(T21="",Q21=""),"",Q21/(T21*Inputs!$B$19))</f>
-        <v/>
-      </c>
-      <c r="V21" s="10">
-        <f>IF(OR(R21="",Q21=""),"",Q21/R21)</f>
-        <v/>
-      </c>
-      <c r="W21" s="10">
-        <f>IF(OR(R21="",T21=""),"",T21/R21)</f>
-        <v/>
-      </c>
-      <c r="X21" s="10">
-        <f>IF(A21="","",IF(OR(UPPER(TRIM(Inputs!$B$15))="MANNING",UPPER(TRIM(Inputs!$B$15))="M"),W21,IF(OR(UPPER(TRIM(Inputs!$B$15))="MAX",UPPER(TRIM(Inputs!$B$15))="X"),MAX(V21,W21),V21)))</f>
-        <v/>
-      </c>
-      <c r="Y21" s="10">
-        <f>IF(A21="","",IF(UPPER(TRIM(B21))="TRENCH",K21*L21*N21,IF(UPPER(TRIM(B21))="SWALE",K21*L21,0)))</f>
-        <v/>
-      </c>
-      <c r="Z21" s="10">
-        <f>IF(OR(Y21="",F21=""),"",Y21*F21)</f>
-        <v/>
-      </c>
-      <c r="AA21" s="3">
-        <f>IF(A21="","",IF(OR(U21&gt;1,AND(X21&lt;&gt;"",X21&lt;Inputs!$B$16),AND(X21&lt;&gt;"",X21&gt;Inputs!$B$17),G21&lt;Inputs!$B$18,AH21="CHECK"),"CHECK","OK"))</f>
-        <v/>
-      </c>
+      <c r="N21" s="8" t="n"/>
+      <c r="O21" s="10" t="n"/>
+      <c r="P21" s="10" t="n"/>
+      <c r="Q21" s="10" t="n"/>
+      <c r="R21" s="10" t="n"/>
+      <c r="S21" s="10" t="n"/>
+      <c r="T21" s="10" t="n"/>
+      <c r="U21" s="10" t="n"/>
+      <c r="V21" s="10" t="n"/>
+      <c r="W21" s="10" t="n"/>
+      <c r="X21" s="10" t="n"/>
+      <c r="Y21" s="10" t="n"/>
+      <c r="Z21" s="10" t="n"/>
+      <c r="AA21" s="3" t="n"/>
       <c r="AB21" s="3" t="n"/>
       <c r="AC21" s="8" t="n"/>
-      <c r="AD21" s="10">
-        <f>IF(A21="","",IF(AC21&lt;&gt;"",AC21,IF(E21="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E21,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),Inputs!$B$57,0),""))))</f>
-        <v/>
-      </c>
-      <c r="AE21" s="10">
-        <f>IF(OR(AD21="",F21="",G21=""),"",AD21+F21*G21)</f>
-        <v/>
-      </c>
-      <c r="AF21" s="10">
-        <f>IF(OR(E21="",A21=""),"",IFERROR(INDEX($AE$4:$AE$204,MATCH(E21,$A$4:$A$204,0)),""))</f>
-        <v/>
-      </c>
-      <c r="AG21" s="10">
-        <f>IF(OR(AD21="",AF21=""),"",AD21-AF21)</f>
-        <v/>
-      </c>
-      <c r="AH21" s="3">
-        <f>IF(A21="","",IF(E21="","TERMINAL",IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),IF(OR(AG21="",AJ21="",AK21=""),"INFO",IF(AND(AG21&gt;=AJ21,AG21&lt;=AK21),"OK","CHECK")),IF(AG21="","INFO",IF(ABS(AG21)&lt;=Inputs!$B$54,"OK","CHECK")))))</f>
-        <v/>
-      </c>
-      <c r="AI21" s="11">
-        <f>IF(A21="","",IF(E21="","",IFERROR(INDEX($B$4:$B$204,MATCH(E21,$A$4:$A$204,0)),"")))</f>
-        <v/>
-      </c>
-      <c r="AJ21" s="11">
-        <f>IF(A21="","",IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),Inputs!$B$55,0))</f>
-        <v/>
-      </c>
-      <c r="AK21" s="11">
-        <f>IF(A21="","",IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),Inputs!$B$56,Inputs!$B$54))</f>
-        <v/>
-      </c>
-      <c r="AL21" s="3">
-        <f>IF(A21="","",IF(E21="","TERMINAL",IF(OR(AND(UPPER(TRIM(B21))="SWALE",UPPER(TRIM(AI21))="PIPE"),AND(UPPER(TRIM(B21))="TRENCH",UPPER(TRIM(AI21))="PIPE")),IF(OR(AG21="",AJ21="",AK21=""),"INFO",IF(AND(AG21&gt;=AJ21,AG21&lt;=AK21),"OK","CHECK")),"N/A")))</f>
-        <v/>
-      </c>
+      <c r="AD21" s="10" t="n"/>
+      <c r="AE21" s="10" t="n"/>
+      <c r="AF21" s="10" t="n"/>
+      <c r="AG21" s="10" t="n"/>
+      <c r="AH21" s="3" t="n"/>
+      <c r="AI21" s="11" t="n"/>
+      <c r="AJ21" s="11" t="n"/>
+      <c r="AK21" s="11" t="n"/>
+      <c r="AL21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -14049,107 +13741,36 @@
       <c r="F22" s="8" t="n"/>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
-      <c r="I22" s="10">
-        <f>IF(A22="","",IF(H22&lt;&gt;"",H22,IF(UPPER(TRIM(B22))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B22))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
-        <v/>
-      </c>
+      <c r="I22" s="10" t="n"/>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="n"/>
       <c r="M22" s="8" t="n"/>
-      <c r="N22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="10">
-        <f>IF(A22="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A22))</f>
-        <v/>
-      </c>
-      <c r="P22" s="10">
-        <f>IF(A22="","",SUMIFS($Q$4:$Q$204,$E$4:$E$204,$A22))</f>
-        <v/>
-      </c>
-      <c r="Q22" s="10">
-        <f>IF(A22="","",(O22+P22)*Inputs!$B$6)</f>
-        <v/>
-      </c>
-      <c r="R22" s="10">
-        <f>IF(A22="","",IF(UPPER(TRIM(B22))="PIPE",PI()*(J22/1000)^2/4,IF(OR(K22="",L22=""),"",L22*(K22+M22*L22))))</f>
-        <v/>
-      </c>
-      <c r="S22" s="10">
-        <f>IF(A22="","",IF(UPPER(TRIM(B22))="PIPE",(J22/1000)/4,IF(OR(R22="",K22="",L22=""),"",R22/(K22+2*L22*SQRT(1+M22^2)))))</f>
-        <v/>
-      </c>
-      <c r="T22" s="10">
-        <f>IF(A22="","",IF(OR(I22="",R22="",S22="",G22=""),"",(1/I22)*R22*(S22^(2/3))*SQRT(G22)))</f>
-        <v/>
-      </c>
-      <c r="U22" s="10">
-        <f>IF(OR(T22="",Q22=""),"",Q22/(T22*Inputs!$B$19))</f>
-        <v/>
-      </c>
-      <c r="V22" s="10">
-        <f>IF(OR(R22="",Q22=""),"",Q22/R22)</f>
-        <v/>
-      </c>
-      <c r="W22" s="10">
-        <f>IF(OR(R22="",T22=""),"",T22/R22)</f>
-        <v/>
-      </c>
-      <c r="X22" s="10">
-        <f>IF(A22="","",IF(OR(UPPER(TRIM(Inputs!$B$15))="MANNING",UPPER(TRIM(Inputs!$B$15))="M"),W22,IF(OR(UPPER(TRIM(Inputs!$B$15))="MAX",UPPER(TRIM(Inputs!$B$15))="X"),MAX(V22,W22),V22)))</f>
-        <v/>
-      </c>
-      <c r="Y22" s="10">
-        <f>IF(A22="","",IF(UPPER(TRIM(B22))="TRENCH",K22*L22*N22,IF(UPPER(TRIM(B22))="SWALE",K22*L22,0)))</f>
-        <v/>
-      </c>
-      <c r="Z22" s="10">
-        <f>IF(OR(Y22="",F22=""),"",Y22*F22)</f>
-        <v/>
-      </c>
-      <c r="AA22" s="3">
-        <f>IF(A22="","",IF(OR(U22&gt;1,AND(X22&lt;&gt;"",X22&lt;Inputs!$B$16),AND(X22&lt;&gt;"",X22&gt;Inputs!$B$17),G22&lt;Inputs!$B$18,AH22="CHECK"),"CHECK","OK"))</f>
-        <v/>
-      </c>
+      <c r="N22" s="8" t="n"/>
+      <c r="O22" s="10" t="n"/>
+      <c r="P22" s="10" t="n"/>
+      <c r="Q22" s="10" t="n"/>
+      <c r="R22" s="10" t="n"/>
+      <c r="S22" s="10" t="n"/>
+      <c r="T22" s="10" t="n"/>
+      <c r="U22" s="10" t="n"/>
+      <c r="V22" s="10" t="n"/>
+      <c r="W22" s="10" t="n"/>
+      <c r="X22" s="10" t="n"/>
+      <c r="Y22" s="10" t="n"/>
+      <c r="Z22" s="10" t="n"/>
+      <c r="AA22" s="3" t="n"/>
       <c r="AB22" s="3" t="n"/>
       <c r="AC22" s="8" t="n"/>
-      <c r="AD22" s="10">
-        <f>IF(A22="","",IF(AC22&lt;&gt;"",AC22,IF(E22="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E22,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),Inputs!$B$57,0),""))))</f>
-        <v/>
-      </c>
-      <c r="AE22" s="10">
-        <f>IF(OR(AD22="",F22="",G22=""),"",AD22+F22*G22)</f>
-        <v/>
-      </c>
-      <c r="AF22" s="10">
-        <f>IF(OR(E22="",A22=""),"",IFERROR(INDEX($AE$4:$AE$204,MATCH(E22,$A$4:$A$204,0)),""))</f>
-        <v/>
-      </c>
-      <c r="AG22" s="10">
-        <f>IF(OR(AD22="",AF22=""),"",AD22-AF22)</f>
-        <v/>
-      </c>
-      <c r="AH22" s="3">
-        <f>IF(A22="","",IF(E22="","TERMINAL",IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),IF(OR(AG22="",AJ22="",AK22=""),"INFO",IF(AND(AG22&gt;=AJ22,AG22&lt;=AK22),"OK","CHECK")),IF(AG22="","INFO",IF(ABS(AG22)&lt;=Inputs!$B$54,"OK","CHECK")))))</f>
-        <v/>
-      </c>
-      <c r="AI22" s="11">
-        <f>IF(A22="","",IF(E22="","",IFERROR(INDEX($B$4:$B$204,MATCH(E22,$A$4:$A$204,0)),"")))</f>
-        <v/>
-      </c>
-      <c r="AJ22" s="11">
-        <f>IF(A22="","",IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),Inputs!$B$55,0))</f>
-        <v/>
-      </c>
-      <c r="AK22" s="11">
-        <f>IF(A22="","",IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),Inputs!$B$56,Inputs!$B$54))</f>
-        <v/>
-      </c>
-      <c r="AL22" s="3">
-        <f>IF(A22="","",IF(E22="","TERMINAL",IF(OR(AND(UPPER(TRIM(B22))="SWALE",UPPER(TRIM(AI22))="PIPE"),AND(UPPER(TRIM(B22))="TRENCH",UPPER(TRIM(AI22))="PIPE")),IF(OR(AG22="",AJ22="",AK22=""),"INFO",IF(AND(AG22&gt;=AJ22,AG22&lt;=AK22),"OK","CHECK")),"N/A")))</f>
-        <v/>
-      </c>
+      <c r="AD22" s="10" t="n"/>
+      <c r="AE22" s="10" t="n"/>
+      <c r="AF22" s="10" t="n"/>
+      <c r="AG22" s="10" t="n"/>
+      <c r="AH22" s="3" t="n"/>
+      <c r="AI22" s="11" t="n"/>
+      <c r="AJ22" s="11" t="n"/>
+      <c r="AK22" s="11" t="n"/>
+      <c r="AL22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -14160,107 +13781,36 @@
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
-      <c r="I23" s="10">
-        <f>IF(A23="","",IF(H23&lt;&gt;"",H23,IF(UPPER(TRIM(B23))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B23))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
-        <v/>
-      </c>
+      <c r="I23" s="10" t="n"/>
       <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="8" t="n"/>
-      <c r="N23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="10">
-        <f>IF(A23="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A23))</f>
-        <v/>
-      </c>
-      <c r="P23" s="10">
-        <f>IF(A23="","",SUMIFS($Q$4:$Q$204,$E$4:$E$204,$A23))</f>
-        <v/>
-      </c>
-      <c r="Q23" s="10">
-        <f>IF(A23="","",(O23+P23)*Inputs!$B$6)</f>
-        <v/>
-      </c>
-      <c r="R23" s="10">
-        <f>IF(A23="","",IF(UPPER(TRIM(B23))="PIPE",PI()*(J23/1000)^2/4,IF(OR(K23="",L23=""),"",L23*(K23+M23*L23))))</f>
-        <v/>
-      </c>
-      <c r="S23" s="10">
-        <f>IF(A23="","",IF(UPPER(TRIM(B23))="PIPE",(J23/1000)/4,IF(OR(R23="",K23="",L23=""),"",R23/(K23+2*L23*SQRT(1+M23^2)))))</f>
-        <v/>
-      </c>
-      <c r="T23" s="10">
-        <f>IF(A23="","",IF(OR(I23="",R23="",S23="",G23=""),"",(1/I23)*R23*(S23^(2/3))*SQRT(G23)))</f>
-        <v/>
-      </c>
-      <c r="U23" s="10">
-        <f>IF(OR(T23="",Q23=""),"",Q23/(T23*Inputs!$B$19))</f>
-        <v/>
-      </c>
-      <c r="V23" s="10">
-        <f>IF(OR(R23="",Q23=""),"",Q23/R23)</f>
-        <v/>
-      </c>
-      <c r="W23" s="10">
-        <f>IF(OR(R23="",T23=""),"",T23/R23)</f>
-        <v/>
-      </c>
-      <c r="X23" s="10">
-        <f>IF(A23="","",IF(OR(UPPER(TRIM(Inputs!$B$15))="MANNING",UPPER(TRIM(Inputs!$B$15))="M"),W23,IF(OR(UPPER(TRIM(Inputs!$B$15))="MAX",UPPER(TRIM(Inputs!$B$15))="X"),MAX(V23,W23),V23)))</f>
-        <v/>
-      </c>
-      <c r="Y23" s="10">
-        <f>IF(A23="","",IF(UPPER(TRIM(B23))="TRENCH",K23*L23*N23,IF(UPPER(TRIM(B23))="SWALE",K23*L23,0)))</f>
-        <v/>
-      </c>
-      <c r="Z23" s="10">
-        <f>IF(OR(Y23="",F23=""),"",Y23*F23)</f>
-        <v/>
-      </c>
-      <c r="AA23" s="3">
-        <f>IF(A23="","",IF(OR(U23&gt;1,AND(X23&lt;&gt;"",X23&lt;Inputs!$B$16),AND(X23&lt;&gt;"",X23&gt;Inputs!$B$17),G23&lt;Inputs!$B$18,AH23="CHECK"),"CHECK","OK"))</f>
-        <v/>
-      </c>
+      <c r="N23" s="8" t="n"/>
+      <c r="O23" s="10" t="n"/>
+      <c r="P23" s="10" t="n"/>
+      <c r="Q23" s="10" t="n"/>
+      <c r="R23" s="10" t="n"/>
+      <c r="S23" s="10" t="n"/>
+      <c r="T23" s="10" t="n"/>
+      <c r="U23" s="10" t="n"/>
+      <c r="V23" s="10" t="n"/>
+      <c r="W23" s="10" t="n"/>
+      <c r="X23" s="10" t="n"/>
+      <c r="Y23" s="10" t="n"/>
+      <c r="Z23" s="10" t="n"/>
+      <c r="AA23" s="3" t="n"/>
       <c r="AB23" s="3" t="n"/>
       <c r="AC23" s="8" t="n"/>
-      <c r="AD23" s="10">
-        <f>IF(A23="","",IF(AC23&lt;&gt;"",AC23,IF(E23="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E23,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),Inputs!$B$57,0),""))))</f>
-        <v/>
-      </c>
-      <c r="AE23" s="10">
-        <f>IF(OR(AD23="",F23="",G23=""),"",AD23+F23*G23)</f>
-        <v/>
-      </c>
-      <c r="AF23" s="10">
-        <f>IF(OR(E23="",A23=""),"",IFERROR(INDEX($AE$4:$AE$204,MATCH(E23,$A$4:$A$204,0)),""))</f>
-        <v/>
-      </c>
-      <c r="AG23" s="10">
-        <f>IF(OR(AD23="",AF23=""),"",AD23-AF23)</f>
-        <v/>
-      </c>
-      <c r="AH23" s="3">
-        <f>IF(A23="","",IF(E23="","TERMINAL",IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),IF(OR(AG23="",AJ23="",AK23=""),"INFO",IF(AND(AG23&gt;=AJ23,AG23&lt;=AK23),"OK","CHECK")),IF(AG23="","INFO",IF(ABS(AG23)&lt;=Inputs!$B$54,"OK","CHECK")))))</f>
-        <v/>
-      </c>
-      <c r="AI23" s="11">
-        <f>IF(A23="","",IF(E23="","",IFERROR(INDEX($B$4:$B$204,MATCH(E23,$A$4:$A$204,0)),"")))</f>
-        <v/>
-      </c>
-      <c r="AJ23" s="11">
-        <f>IF(A23="","",IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),Inputs!$B$55,0))</f>
-        <v/>
-      </c>
-      <c r="AK23" s="11">
-        <f>IF(A23="","",IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),Inputs!$B$56,Inputs!$B$54))</f>
-        <v/>
-      </c>
-      <c r="AL23" s="3">
-        <f>IF(A23="","",IF(E23="","TERMINAL",IF(OR(AND(UPPER(TRIM(B23))="SWALE",UPPER(TRIM(AI23))="PIPE"),AND(UPPER(TRIM(B23))="TRENCH",UPPER(TRIM(AI23))="PIPE")),IF(OR(AG23="",AJ23="",AK23=""),"INFO",IF(AND(AG23&gt;=AJ23,AG23&lt;=AK23),"OK","CHECK")),"N/A")))</f>
-        <v/>
-      </c>
+      <c r="AD23" s="10" t="n"/>
+      <c r="AE23" s="10" t="n"/>
+      <c r="AF23" s="10" t="n"/>
+      <c r="AG23" s="10" t="n"/>
+      <c r="AH23" s="3" t="n"/>
+      <c r="AI23" s="11" t="n"/>
+      <c r="AJ23" s="11" t="n"/>
+      <c r="AK23" s="11" t="n"/>
+      <c r="AL23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -14271,107 +13821,36 @@
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
-      <c r="I24" s="10">
-        <f>IF(A24="","",IF(H24&lt;&gt;"",H24,IF(UPPER(TRIM(B24))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B24))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
-        <v/>
-      </c>
+      <c r="I24" s="10" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="n"/>
       <c r="M24" s="8" t="n"/>
-      <c r="N24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="10">
-        <f>IF(A24="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A24))</f>
-        <v/>
-      </c>
-      <c r="P24" s="10">
-        <f>IF(A24="","",SUMIFS($Q$4:$Q$204,$E$4:$E$204,$A24))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="10">
-        <f>IF(A24="","",(O24+P24)*Inputs!$B$6)</f>
-        <v/>
-      </c>
-      <c r="R24" s="10">
-        <f>IF(A24="","",IF(UPPER(TRIM(B24))="PIPE",PI()*(J24/1000)^2/4,IF(OR(K24="",L24=""),"",L24*(K24+M24*L24))))</f>
-        <v/>
-      </c>
-      <c r="S24" s="10">
-        <f>IF(A24="","",IF(UPPER(TRIM(B24))="PIPE",(J24/1000)/4,IF(OR(R24="",K24="",L24=""),"",R24/(K24+2*L24*SQRT(1+M24^2)))))</f>
-        <v/>
-      </c>
-      <c r="T24" s="10">
-        <f>IF(A24="","",IF(OR(I24="",R24="",S24="",G24=""),"",(1/I24)*R24*(S24^(2/3))*SQRT(G24)))</f>
-        <v/>
-      </c>
-      <c r="U24" s="10">
-        <f>IF(OR(T24="",Q24=""),"",Q24/(T24*Inputs!$B$19))</f>
-        <v/>
-      </c>
-      <c r="V24" s="10">
-        <f>IF(OR(R24="",Q24=""),"",Q24/R24)</f>
-        <v/>
-      </c>
-      <c r="W24" s="10">
-        <f>IF(OR(R24="",T24=""),"",T24/R24)</f>
-        <v/>
-      </c>
-      <c r="X24" s="10">
-        <f>IF(A24="","",IF(OR(UPPER(TRIM(Inputs!$B$15))="MANNING",UPPER(TRIM(Inputs!$B$15))="M"),W24,IF(OR(UPPER(TRIM(Inputs!$B$15))="MAX",UPPER(TRIM(Inputs!$B$15))="X"),MAX(V24,W24),V24)))</f>
-        <v/>
-      </c>
-      <c r="Y24" s="10">
-        <f>IF(A24="","",IF(UPPER(TRIM(B24))="TRENCH",K24*L24*N24,IF(UPPER(TRIM(B24))="SWALE",K24*L24,0)))</f>
-        <v/>
-      </c>
-      <c r="Z24" s="10">
-        <f>IF(OR(Y24="",F24=""),"",Y24*F24)</f>
-        <v/>
-      </c>
-      <c r="AA24" s="3">
-        <f>IF(A24="","",IF(OR(U24&gt;1,AND(X24&lt;&gt;"",X24&lt;Inputs!$B$16),AND(X24&lt;&gt;"",X24&gt;Inputs!$B$17),G24&lt;Inputs!$B$18,AH24="CHECK"),"CHECK","OK"))</f>
-        <v/>
-      </c>
+      <c r="N24" s="8" t="n"/>
+      <c r="O24" s="10" t="n"/>
+      <c r="P24" s="10" t="n"/>
+      <c r="Q24" s="10" t="n"/>
+      <c r="R24" s="10" t="n"/>
+      <c r="S24" s="10" t="n"/>
+      <c r="T24" s="10" t="n"/>
+      <c r="U24" s="10" t="n"/>
+      <c r="V24" s="10" t="n"/>
+      <c r="W24" s="10" t="n"/>
+      <c r="X24" s="10" t="n"/>
+      <c r="Y24" s="10" t="n"/>
+      <c r="Z24" s="10" t="n"/>
+      <c r="AA24" s="3" t="n"/>
       <c r="AB24" s="3" t="n"/>
       <c r="AC24" s="8" t="n"/>
-      <c r="AD24" s="10">
-        <f>IF(A24="","",IF(AC24&lt;&gt;"",AC24,IF(E24="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E24,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),Inputs!$B$57,0),""))))</f>
-        <v/>
-      </c>
-      <c r="AE24" s="10">
-        <f>IF(OR(AD24="",F24="",G24=""),"",AD24+F24*G24)</f>
-        <v/>
-      </c>
-      <c r="AF24" s="10">
-        <f>IF(OR(E24="",A24=""),"",IFERROR(INDEX($AE$4:$AE$204,MATCH(E24,$A$4:$A$204,0)),""))</f>
-        <v/>
-      </c>
-      <c r="AG24" s="10">
-        <f>IF(OR(AD24="",AF24=""),"",AD24-AF24)</f>
-        <v/>
-      </c>
-      <c r="AH24" s="3">
-        <f>IF(A24="","",IF(E24="","TERMINAL",IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),IF(OR(AG24="",AJ24="",AK24=""),"INFO",IF(AND(AG24&gt;=AJ24,AG24&lt;=AK24),"OK","CHECK")),IF(AG24="","INFO",IF(ABS(AG24)&lt;=Inputs!$B$54,"OK","CHECK")))))</f>
-        <v/>
-      </c>
-      <c r="AI24" s="11">
-        <f>IF(A24="","",IF(E24="","",IFERROR(INDEX($B$4:$B$204,MATCH(E24,$A$4:$A$204,0)),"")))</f>
-        <v/>
-      </c>
-      <c r="AJ24" s="11">
-        <f>IF(A24="","",IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),Inputs!$B$55,0))</f>
-        <v/>
-      </c>
-      <c r="AK24" s="11">
-        <f>IF(A24="","",IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),Inputs!$B$56,Inputs!$B$54))</f>
-        <v/>
-      </c>
-      <c r="AL24" s="3">
-        <f>IF(A24="","",IF(E24="","TERMINAL",IF(OR(AND(UPPER(TRIM(B24))="SWALE",UPPER(TRIM(AI24))="PIPE"),AND(UPPER(TRIM(B24))="TRENCH",UPPER(TRIM(AI24))="PIPE")),IF(OR(AG24="",AJ24="",AK24=""),"INFO",IF(AND(AG24&gt;=AJ24,AG24&lt;=AK24),"OK","CHECK")),"N/A")))</f>
-        <v/>
-      </c>
+      <c r="AD24" s="10" t="n"/>
+      <c r="AE24" s="10" t="n"/>
+      <c r="AF24" s="10" t="n"/>
+      <c r="AG24" s="10" t="n"/>
+      <c r="AH24" s="3" t="n"/>
+      <c r="AI24" s="11" t="n"/>
+      <c r="AJ24" s="11" t="n"/>
+      <c r="AK24" s="11" t="n"/>
+      <c r="AL24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -14382,107 +13861,36 @@
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
-      <c r="I25" s="10">
-        <f>IF(A25="","",IF(H25&lt;&gt;"",H25,IF(UPPER(TRIM(B25))="PIPE",Inputs!$B$7,IF(UPPER(TRIM(B25))="SWALE",Inputs!$B$8,Inputs!$B$9))))</f>
-        <v/>
-      </c>
+      <c r="I25" s="10" t="n"/>
       <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="8" t="n"/>
-      <c r="N25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="10">
-        <f>IF(A25="","",SUMIFS(Zones_tributaires!$I:$I,Zones_tributaires!$J:$J,$A25))</f>
-        <v/>
-      </c>
-      <c r="P25" s="10">
-        <f>IF(A25="","",SUMIFS($Q$4:$Q$204,$E$4:$E$204,$A25))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="10">
-        <f>IF(A25="","",(O25+P25)*Inputs!$B$6)</f>
-        <v/>
-      </c>
-      <c r="R25" s="10">
-        <f>IF(A25="","",IF(UPPER(TRIM(B25))="PIPE",PI()*(J25/1000)^2/4,IF(OR(K25="",L25=""),"",L25*(K25+M25*L25))))</f>
-        <v/>
-      </c>
-      <c r="S25" s="10">
-        <f>IF(A25="","",IF(UPPER(TRIM(B25))="PIPE",(J25/1000)/4,IF(OR(R25="",K25="",L25=""),"",R25/(K25+2*L25*SQRT(1+M25^2)))))</f>
-        <v/>
-      </c>
-      <c r="T25" s="10">
-        <f>IF(A25="","",IF(OR(I25="",R25="",S25="",G25=""),"",(1/I25)*R25*(S25^(2/3))*SQRT(G25)))</f>
-        <v/>
-      </c>
-      <c r="U25" s="10">
-        <f>IF(OR(T25="",Q25=""),"",Q25/(T25*Inputs!$B$19))</f>
-        <v/>
-      </c>
-      <c r="V25" s="10">
-        <f>IF(OR(R25="",Q25=""),"",Q25/R25)</f>
-        <v/>
-      </c>
-      <c r="W25" s="10">
-        <f>IF(OR(R25="",T25=""),"",T25/R25)</f>
-        <v/>
-      </c>
-      <c r="X25" s="10">
-        <f>IF(A25="","",IF(OR(UPPER(TRIM(Inputs!$B$15))="MANNING",UPPER(TRIM(Inputs!$B$15))="M"),W25,IF(OR(UPPER(TRIM(Inputs!$B$15))="MAX",UPPER(TRIM(Inputs!$B$15))="X"),MAX(V25,W25),V25)))</f>
-        <v/>
-      </c>
-      <c r="Y25" s="10">
-        <f>IF(A25="","",IF(UPPER(TRIM(B25))="TRENCH",K25*L25*N25,IF(UPPER(TRIM(B25))="SWALE",K25*L25,0)))</f>
-        <v/>
-      </c>
-      <c r="Z25" s="10">
-        <f>IF(OR(Y25="",F25=""),"",Y25*F25)</f>
-        <v/>
-      </c>
-      <c r="AA25" s="3">
-        <f>IF(A25="","",IF(OR(U25&gt;1,AND(X25&lt;&gt;"",X25&lt;Inputs!$B$16),AND(X25&lt;&gt;"",X25&gt;Inputs!$B$17),G25&lt;Inputs!$B$18,AH25="CHECK"),"CHECK","OK"))</f>
-        <v/>
-      </c>
+      <c r="N25" s="8" t="n"/>
+      <c r="O25" s="10" t="n"/>
+      <c r="P25" s="10" t="n"/>
+      <c r="Q25" s="10" t="n"/>
+      <c r="R25" s="10" t="n"/>
+      <c r="S25" s="10" t="n"/>
+      <c r="T25" s="10" t="n"/>
+      <c r="U25" s="10" t="n"/>
+      <c r="V25" s="10" t="n"/>
+      <c r="W25" s="10" t="n"/>
+      <c r="X25" s="10" t="n"/>
+      <c r="Y25" s="10" t="n"/>
+      <c r="Z25" s="10" t="n"/>
+      <c r="AA25" s="3" t="n"/>
       <c r="AB25" s="3" t="n"/>
       <c r="AC25" s="8" t="n"/>
-      <c r="AD25" s="10">
-        <f>IF(A25="","",IF(AC25&lt;&gt;"",AC25,IF(E25="",Inputs!$B$38,IFERROR(INDEX($AE$4:$AE$204,MATCH(E25,$A$4:$A$204,0))+IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),Inputs!$B$57,0),""))))</f>
-        <v/>
-      </c>
-      <c r="AE25" s="10">
-        <f>IF(OR(AD25="",F25="",G25=""),"",AD25+F25*G25)</f>
-        <v/>
-      </c>
-      <c r="AF25" s="10">
-        <f>IF(OR(E25="",A25=""),"",IFERROR(INDEX($AE$4:$AE$204,MATCH(E25,$A$4:$A$204,0)),""))</f>
-        <v/>
-      </c>
-      <c r="AG25" s="10">
-        <f>IF(OR(AD25="",AF25=""),"",AD25-AF25)</f>
-        <v/>
-      </c>
-      <c r="AH25" s="3">
-        <f>IF(A25="","",IF(E25="","TERMINAL",IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),IF(OR(AG25="",AJ25="",AK25=""),"INFO",IF(AND(AG25&gt;=AJ25,AG25&lt;=AK25),"OK","CHECK")),IF(AG25="","INFO",IF(ABS(AG25)&lt;=Inputs!$B$54,"OK","CHECK")))))</f>
-        <v/>
-      </c>
-      <c r="AI25" s="11">
-        <f>IF(A25="","",IF(E25="","",IFERROR(INDEX($B$4:$B$204,MATCH(E25,$A$4:$A$204,0)),"")))</f>
-        <v/>
-      </c>
-      <c r="AJ25" s="11">
-        <f>IF(A25="","",IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),Inputs!$B$55,0))</f>
-        <v/>
-      </c>
-      <c r="AK25" s="11">
-        <f>IF(A25="","",IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),Inputs!$B$56,Inputs!$B$54))</f>
-        <v/>
-      </c>
-      <c r="AL25" s="3">
-        <f>IF(A25="","",IF(E25="","TERMINAL",IF(OR(AND(UPPER(TRIM(B25))="SWALE",UPPER(TRIM(AI25))="PIPE"),AND(UPPER(TRIM(B25))="TRENCH",UPPER(TRIM(AI25))="PIPE")),IF(OR(AG25="",AJ25="",AK25=""),"INFO",IF(AND(AG25&gt;=AJ25,AG25&lt;=AK25),"OK","CHECK")),"N/A")))</f>
-        <v/>
-      </c>
+      <c r="AD25" s="10" t="n"/>
+      <c r="AE25" s="10" t="n"/>
+      <c r="AF25" s="10" t="n"/>
+      <c r="AG25" s="10" t="n"/>
+      <c r="AH25" s="3" t="n"/>
+      <c r="AI25" s="11" t="n"/>
+      <c r="AJ25" s="11" t="n"/>
+      <c r="AK25" s="11" t="n"/>
+      <c r="AL25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -34412,7 +33820,7 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>NOEUDS / OUVRAGES - CAPACITE DE STOCKAGE TAMPON</t>
+          <t>NOEUDS — modèle simplifié (plan 1796-C-03)</t>
         </is>
       </c>
     </row>
@@ -34464,7 +33872,7 @@
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Buffer_time_min</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -34486,19 +33894,19 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SWALE_NODE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>23.97</v>
+        <v>23.46</v>
       </c>
       <c r="D4" s="8">
-        <f>C4-0.3</f>
+        <f>C4-1</f>
         <v/>
       </c>
       <c r="E4" s="10">
@@ -34507,22 +33915,21 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>CIRC</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>9.6</v>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="H4" s="8" t="n"/>
       <c r="I4" s="10">
         <f>IF(A4="","",IF(UPPER(TRIM(F4))="CIRC",PI()*(G4/2)^2*E4,IF(UPPER(TRIM(F4))="RECT",G4*H4*E4,"")))</f>
         <v/>
       </c>
-      <c r="J4" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>CB ouest — reçoit gazon+pavé ouest</t>
+        </is>
       </c>
       <c r="K4" s="10">
         <f>IF(A4="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A4))</f>
@@ -34540,20 +33947,19 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>SWALE_NODE</t>
+          <t>CB</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>23.91</v>
-      </c>
-      <c r="D5" s="8">
-        <f>C5-0.3</f>
-        <v/>
+        <v>23.5</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>21.66</v>
       </c>
       <c r="E5" s="10">
         <f>IF(OR(C5="",D5=""),"",MAX(0,C5-D5))</f>
@@ -34561,22 +33967,21 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>CIRC</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>9.699999999999999</v>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="H5" s="8" t="n"/>
       <c r="I5" s="10">
         <f>IF(A5="","",IF(UPPER(TRIM(F5))="CIRC",PI()*(G5/2)^2*E5,IF(UPPER(TRIM(F5))="RECT",G5*H5*E5,"")))</f>
         <v/>
       </c>
-      <c r="J5" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>CB est sud — reçoit bande arbres + sud-est</t>
+        </is>
       </c>
       <c r="K5" s="10">
         <f>IF(A5="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A5))</f>
@@ -34594,20 +33999,19 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>RP-02</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>23.67</v>
-      </c>
-      <c r="D6" s="8">
-        <f>C6-0.3</f>
-        <v/>
+        <v>22.82</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>21.62</v>
       </c>
       <c r="E6" s="10">
         <f>IF(OR(C6="",D6=""),"",MAX(0,C6-D6))</f>
@@ -34615,20 +34019,21 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>CIRC</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
-        <v>0.2</v>
+        <v>1.2</v>
       </c>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="10">
         <f>IF(A6="","",IF(UPPER(TRIM(F6))="CIRC",PI()*(G6/2)^2*E6,IF(UPPER(TRIM(F6))="RECT",G6*H6*E6,"")))</f>
         <v/>
       </c>
-      <c r="J6" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Regard — fusion ouest+est vers rue</t>
+        </is>
       </c>
       <c r="K6" s="10">
         <f>IF(A6="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A6))</f>
@@ -34646,20 +34051,16 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>J-SUD-EST</t>
+          <t>RS-EX</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>23.2</v>
-      </c>
+          <t>EXIST</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="10">
         <f>IF(OR(C7="",D7=""),"",MAX(0,C7-D7))</f>
         <v/>
@@ -34670,16 +34071,17 @@
         </is>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.2</v>
+        <v>1.05</v>
       </c>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="10">
         <f>IF(A7="","",IF(UPPER(TRIM(F7))="CIRC",PI()*(G7/2)^2*E7,IF(UPPER(TRIM(F7))="RECT",G7*H7*E7,"")))</f>
         <v/>
       </c>
-      <c r="J7" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Réseau pluvial existant (rue)</t>
+        </is>
       </c>
       <c r="K7" s="10">
         <f>IF(A7="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A7))</f>
@@ -34697,19 +34099,20 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>J-SUD-OUEST</t>
+          <t>MEC-OUT</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>23.05</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>23.05</v>
+        <v>23.63</v>
+      </c>
+      <c r="D8" s="8">
+        <f>C8-1</f>
+        <v/>
       </c>
       <c r="E8" s="10">
         <f>IF(OR(C8="",D8=""),"",MAX(0,C8-D8))</f>
@@ -34717,22 +34120,21 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>CIRC</t>
         </is>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>10.619</v>
-      </c>
+        <v>0.3</v>
+      </c>
+      <c r="H8" s="8" t="n"/>
       <c r="I8" s="10">
         <f>IF(A8="","",IF(UPPER(TRIM(F8))="CIRC",PI()*(G8/2)^2*E8,IF(UPPER(TRIM(F8))="RECT",G8*H8*E8,"")))</f>
         <v/>
       </c>
-      <c r="J8" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Sortie mécanique bâtiment (toit/tréfond)</t>
+        </is>
       </c>
       <c r="K8" s="10">
         <f>IF(A8="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A8))</f>
@@ -34750,19 +34152,19 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>P-W1</t>
+          <t>BASSIN-RET</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RETENTION</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>23.58</v>
+        <v>23.56</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>22.58</v>
+        <v>21.62</v>
       </c>
       <c r="E9" s="10">
         <f>IF(OR(C9="",D9=""),"",MAX(0,C9-D9))</f>
@@ -34770,22 +34172,25 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>3</v>
+          <t>RECT</t>
+        </is>
+      </c>
+      <c r="G9" s="8">
+        <f>Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="H9" s="8">
+        <f>Inputs!$B$35</f>
+        <v/>
       </c>
       <c r="I9" s="10">
         <f>IF(A9="","",IF(UPPER(TRIM(F9))="CIRC",PI()*(G9/2)^2*E9,IF(UPPER(TRIM(F9))="RECT",G9*H9*E9,"")))</f>
         <v/>
       </c>
-      <c r="J9" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Bassin rétention EZ-STORM</t>
+        </is>
       </c>
       <c r="K9" s="10">
         <f>IF(A9="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A9))</f>
@@ -34803,16 +34208,16 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>P-W2</t>
+          <t>BANDE_ARBRES</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>SWALE_NODE</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>23.667</v>
+        <v>23.9</v>
       </c>
       <c r="D10" s="8">
         <f>C10-1</f>
@@ -34824,20 +34229,23 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>CIRC</t>
+          <t>RECT</t>
         </is>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H10" s="8" t="n"/>
+        <v>2.5</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>20</v>
+      </c>
       <c r="I10" s="10">
         <f>IF(A10="","",IF(UPPER(TRIM(F10))="CIRC",PI()*(G10/2)^2*E10,IF(UPPER(TRIM(F10))="RECT",G10*H10*E10,"")))</f>
         <v/>
       </c>
-      <c r="J10" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Noeud conceptuel bande arbres (pas de CB)</t>
+        </is>
       </c>
       <c r="K10" s="10">
         <f>IF(A10="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A10))</f>
@@ -34853,35 +34261,16 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>P-W3</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>23.556</v>
-      </c>
-      <c r="D11" s="8">
-        <f>C11-1</f>
-        <v/>
-      </c>
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="10">
         <f>IF(OR(C11="",D11=""),"",MAX(0,C11-D11))</f>
         <v/>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="10">
         <f>IF(A11="","",IF(UPPER(TRIM(F11))="CIRC",PI()*(G11/2)^2*E11,IF(UPPER(TRIM(F11))="RECT",G11*H11*E11,"")))</f>
@@ -34905,35 +34294,16 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>P-W4</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>23.504</v>
-      </c>
-      <c r="D12" s="8">
-        <f>C12-1</f>
-        <v/>
-      </c>
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="10">
         <f>IF(OR(C12="",D12=""),"",MAX(0,C12-D12))</f>
         <v/>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="10">
         <f>IF(A12="","",IF(UPPER(TRIM(F12))="CIRC",PI()*(G12/2)^2*E12,IF(UPPER(TRIM(F12))="RECT",G12*H12*E12,"")))</f>
@@ -34957,35 +34327,16 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>P-W5</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="D13" s="8">
-        <f>C13-1</f>
-        <v/>
-      </c>
+      <c r="A13" s="3" t="n"/>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="10">
         <f>IF(OR(C13="",D13=""),"",MAX(0,C13-D13))</f>
         <v/>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="10">
         <f>IF(A13="","",IF(UPPER(TRIM(F13))="CIRC",PI()*(G13/2)^2*E13,IF(UPPER(TRIM(F13))="RECT",G13*H13*E13,"")))</f>
@@ -35009,35 +34360,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>P-W6</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="D14" s="8">
-        <f>C14-1</f>
-        <v/>
-      </c>
+      <c r="A14" s="3" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="10">
         <f>IF(OR(C14="",D14=""),"",MAX(0,C14-D14))</f>
         <v/>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="10">
         <f>IF(A14="","",IF(UPPER(TRIM(F14))="CIRC",PI()*(G14/2)^2*E14,IF(UPPER(TRIM(F14))="RECT",G14*H14*E14,"")))</f>
@@ -35061,35 +34393,16 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-EST</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n">
-        <v>23.63</v>
-      </c>
-      <c r="D15" s="8">
-        <f>C15-1</f>
-        <v/>
-      </c>
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="10">
         <f>IF(OR(C15="",D15=""),"",MAX(0,C15-D15))</f>
         <v/>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="10">
         <f>IF(A15="","",IF(UPPER(TRIM(F15))="CIRC",PI()*(G15/2)^2*E15,IF(UPPER(TRIM(F15))="RECT",G15*H15*E15,"")))</f>
@@ -35113,39 +34426,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>RETENTION</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>23.56</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>21.62</v>
-      </c>
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="10">
         <f>IF(OR(C16="",D16=""),"",MAX(0,C16-D16))</f>
         <v/>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>RECT</t>
-        </is>
-      </c>
-      <c r="G16" s="8">
-        <f>Inputs!$B$34</f>
-        <v/>
-      </c>
-      <c r="H16" s="8">
-        <f>Inputs!$B$35</f>
-        <v/>
-      </c>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
       <c r="I16" s="10">
         <f>IF(A16="","",IF(UPPER(TRIM(F16))="CIRC",PI()*(G16/2)^2*E16,IF(UPPER(TRIM(F16))="RECT",G16*H16*E16,"")))</f>
         <v/>
@@ -35167,30 +34458,16 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
+      <c r="A17" s="3" t="n"/>
+      <c r="B17" s="3" t="n"/>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="10">
         <f>IF(OR(C17="",D17=""),"",MAX(0,C17-D17))</f>
         <v/>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>1.2</v>
-      </c>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="10">
         <f>IF(A17="","",IF(UPPER(TRIM(F17))="CIRC",PI()*(G17/2)^2*E17,IF(UPPER(TRIM(F17))="RECT",G17*H17*E17,"")))</f>
@@ -35214,30 +34491,16 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>P-011</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="3" t="n"/>
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="10">
         <f>IF(OR(C18="",D18=""),"",MAX(0,C18-D18))</f>
         <v/>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>0.3</v>
-      </c>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
       <c r="H18" s="8" t="n"/>
       <c r="I18" s="10">
         <f>IF(A18="","",IF(UPPER(TRIM(F18))="CIRC",PI()*(G18/2)^2*E18,IF(UPPER(TRIM(F18))="RECT",G18*H18*E18,"")))</f>
@@ -35261,34 +34524,16 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>RP-02</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="n">
-        <v>23.64</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>21.62</v>
-      </c>
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
       <c r="E19" s="10">
         <f>IF(OR(C19="",D19=""),"",MAX(0,C19-D19))</f>
         <v/>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>CIRC</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>0.3</v>
-      </c>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="10">
         <f>IF(A19="","",IF(UPPER(TRIM(F19))="CIRC",PI()*(G19/2)^2*E19,IF(UPPER(TRIM(F19))="RECT",G19*H19*E19,"")))</f>
@@ -41356,14 +40601,14 @@
     <row r="1">
       <c r="A1" s="40" t="inlineStr">
         <is>
-          <t>CONVENTION DE NOMMAGE — plan PDF 1796-C-03-Model</t>
+          <t>NOMMAGE SIMPLIFIÉ — plan 1796-C-03</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" s="22">
       <c r="A2" s="41" t="inlineStr">
         <is>
-          <t>Element_ID (E01…) = clé des débits (Zones!J et Elements!O). P-xx / RP-02 / MH-… = noeuds From/To. Ne pas mettre un noeud dans Zones!J.</t>
+          <t>Element_ID lisible = clé Zones!J = Elements!A. Nodes = P-03, P-07, RP-02, etc.</t>
         </is>
       </c>
     </row>
@@ -41377,12 +40622,12 @@
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
-          <t>Plan_PDF</t>
+          <t>Plan</t>
         </is>
       </c>
       <c r="B4" s="31" t="inlineStr">
         <is>
-          <t>Node_ID_modele</t>
+          <t>Dans le modèle</t>
         </is>
       </c>
       <c r="C4" s="31" t="inlineStr">
@@ -41392,7 +40637,7 @@
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>Element(s) liés</t>
+          <t>Lié à</t>
         </is>
       </c>
       <c r="E4" s="31" t="inlineStr">
@@ -41404,12 +40649,12 @@
     <row r="5">
       <c r="A5" s="42" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="B5" s="42" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>P-03</t>
         </is>
       </c>
       <c r="C5" s="42" t="inlineStr">
@@ -41419,24 +40664,24 @@
       </c>
       <c r="D5" s="42" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>OUEST_P03_RP02</t>
         </is>
       </c>
       <c r="E5" s="42" t="inlineStr">
         <is>
-          <t>CB bande est amont</t>
+          <t>Catchbasin OUEST — gazon + pavage</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="B6" s="42" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-07</t>
         </is>
       </c>
       <c r="C6" s="42" t="inlineStr">
@@ -41446,419 +40691,219 @@
       </c>
       <c r="D6" s="42" t="inlineStr">
         <is>
-          <t>E01/E02</t>
+          <t>EST_P07_RP02</t>
         </is>
       </c>
       <c r="E6" s="42" t="inlineStr">
         <is>
-          <t>CB est intermédiaire</t>
+          <t>Catchbasin EST sud — seul CB est</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="42" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>RP-02</t>
         </is>
       </c>
       <c r="B7" s="42" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>RP-02</t>
         </is>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
         <is>
-          <t>E02/E03</t>
+          <t>RP02_VERS_RUE</t>
         </is>
       </c>
       <c r="E7" s="42" t="inlineStr">
         <is>
-          <t>CB est aval → pipe bassin</t>
+          <t>Regard fusion → rue</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>P-04</t>
+          <t>RS-EX</t>
         </is>
       </c>
       <c r="B8" s="42" t="inlineStr">
         <is>
-          <t>P-04</t>
+          <t>RS-EX</t>
         </is>
       </c>
       <c r="C8" s="42" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>EXIST</t>
         </is>
       </c>
       <c r="D8" s="42" t="inlineStr">
         <is>
-          <t>sud plan</t>
+          <t>aval RP-02</t>
         </is>
       </c>
       <c r="E8" s="42" t="inlineStr">
         <is>
-          <t>CB sud corridor exutoire (plan)</t>
+          <t>Réseau existant</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="42" t="inlineStr">
         <is>
-          <t>P-05</t>
+          <t>Bassin</t>
         </is>
       </c>
       <c r="B9" s="42" t="inlineStr">
         <is>
-          <t>P-05</t>
+          <t>BASSIN-RET</t>
         </is>
       </c>
       <c r="C9" s="42" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>RETENTION</t>
         </is>
       </c>
       <c r="D9" s="42" t="inlineStr">
         <is>
-          <t>sud plan</t>
+          <t>MEC_…_BASSIN</t>
         </is>
       </c>
       <c r="E9" s="42" t="inlineStr">
         <is>
-          <t>CB sud (plan)</t>
+          <t>Rétention sud (toit/tréfond)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="42" t="inlineStr">
         <is>
-          <t>P-06</t>
+          <t>Arbres (jaune)</t>
         </is>
       </c>
       <c r="B10" s="42" t="inlineStr">
         <is>
-          <t>P-06</t>
+          <t>BANDE_ARBRES</t>
         </is>
       </c>
       <c r="C10" s="42" t="inlineStr">
         <is>
-          <t>CB</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D10" s="42" t="inlineStr">
         <is>
-          <t>sud plan</t>
+          <t>EST_ARBRES_VERS_P07</t>
         </is>
       </c>
       <c r="E10" s="42" t="inlineStr">
         <is>
-          <t>CB sud (plan)</t>
+          <t>Pas de CB; seulement arbres</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
         <is>
-          <t>P-07</t>
+          <t>Mécanique</t>
         </is>
       </c>
       <c r="B11" s="42" t="inlineStr">
         <is>
-          <t>P-07</t>
+          <t>MEC-OUT</t>
         </is>
       </c>
       <c r="C11" s="42" t="inlineStr">
         <is>
-          <t>CB/MH</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="D11" s="42" t="inlineStr">
         <is>
-          <t>mécanique est</t>
+          <t>MEC_TOIT_TRESFOND_BASSIN</t>
         </is>
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>Plan: Ø300 vers sud</t>
+          <t>Sortie interne bâtiment</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>P-08</t>
-        </is>
-      </c>
-      <c r="B12" s="42" t="inlineStr">
-        <is>
-          <t>P-08</t>
-        </is>
-      </c>
-      <c r="C12" s="42" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D12" s="42" t="inlineStr">
-        <is>
-          <t>mécanique</t>
-        </is>
-      </c>
-      <c r="E12" s="42" t="inlineStr">
-        <is>
-          <t>Plan: D≈23.52 S VOIR MEC</t>
-        </is>
-      </c>
+      <c r="A12" s="42" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="42" t="n"/>
+      <c r="D12" s="42" t="n"/>
+      <c r="E12" s="42" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>P-09</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>P-09</t>
-        </is>
-      </c>
-      <c r="C13" s="42" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>mécanique</t>
-        </is>
-      </c>
-      <c r="E13" s="42" t="inlineStr">
-        <is>
-          <t>Plan: limite tréfond</t>
-        </is>
-      </c>
+      <c r="A13" s="42" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="42" t="n"/>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>P-011</t>
-        </is>
-      </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>P-011</t>
-        </is>
-      </c>
-      <c r="C14" s="42" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="D14" s="42" t="inlineStr">
-        <is>
-          <t>E09</t>
-        </is>
-      </c>
-      <c r="E14" s="42" t="inlineStr">
-        <is>
-          <t>Limite toiture / sortie MEC (ex J-MECH-OUT)</t>
-        </is>
-      </c>
+      <c r="A14" s="42" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="42" t="n"/>
+      <c r="E14" s="42" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>CAN-010</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>CAN-010</t>
-        </is>
-      </c>
-      <c r="C15" s="42" t="inlineStr">
-        <is>
-          <t>CAN</t>
-        </is>
-      </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>mécanique</t>
-        </is>
-      </c>
-      <c r="E15" s="42" t="inlineStr">
-        <is>
-          <t>Collecteur interne plan</t>
-        </is>
-      </c>
+      <c r="A15" s="42" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="42" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>RP-02</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>RP-02</t>
-        </is>
-      </c>
-      <c r="C16" s="42" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="D16" s="42" t="inlineStr">
-        <is>
-          <t>E08</t>
-        </is>
-      </c>
-      <c r="E16" s="42" t="inlineStr">
-        <is>
-          <t>Regard raccordement (ex J-MH)</t>
-        </is>
-      </c>
+      <c r="A16" s="42" t="n"/>
+      <c r="B16" s="42" t="n"/>
+      <c r="C16" s="42" t="n"/>
+      <c r="D16" s="42" t="n"/>
+      <c r="E16" s="42" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>RP-EX / RS-EX</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="42" t="inlineStr">
-        <is>
-          <t>EXIST</t>
-        </is>
-      </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="42" t="inlineStr">
-        <is>
-          <t>Existant Avenue Dorval</t>
-        </is>
-      </c>
+      <c r="A17" s="42" t="n"/>
+      <c r="B17" s="42" t="n"/>
+      <c r="C17" s="42" t="n"/>
+      <c r="D17" s="42" t="n"/>
+      <c r="E17" s="42" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="42" t="inlineStr">
-        <is>
-          <t>BASSIN RÉTENTION</t>
-        </is>
-      </c>
-      <c r="B18" s="42" t="inlineStr">
-        <is>
-          <t>BASSIN-RET</t>
-        </is>
-      </c>
-      <c r="C18" s="42" t="inlineStr">
-        <is>
-          <t>RETENTION</t>
-        </is>
-      </c>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>E07,E08,E09</t>
-        </is>
-      </c>
-      <c r="E18" s="42" t="inlineStr">
-        <is>
-          <t>EZ-STORM; radier 21.62; Vol≈85 m³</t>
-        </is>
-      </c>
+      <c r="A18" s="42" t="n"/>
+      <c r="B18" s="42" t="n"/>
+      <c r="C18" s="42" t="n"/>
+      <c r="D18" s="42" t="n"/>
+      <c r="E18" s="42" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="42" t="inlineStr">
-        <is>
-          <t>Entrée est bassin</t>
-        </is>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-EST</t>
-        </is>
-      </c>
-      <c r="C19" s="42" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>E03/E07</t>
-        </is>
-      </c>
-      <c r="E19" s="42" t="inlineStr">
-        <is>
-          <t>ex J-BASSIN-IN</t>
-        </is>
-      </c>
+      <c r="A19" s="42" t="n"/>
+      <c r="B19" s="42" t="n"/>
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="42" t="n"/>
+      <c r="E19" s="42" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="42" t="inlineStr">
-        <is>
-          <t>Entrée ouest bassin</t>
-        </is>
-      </c>
-      <c r="B20" s="42" t="inlineStr">
-        <is>
-          <t>MH-BASSIN-OUEST</t>
-        </is>
-      </c>
-      <c r="C20" s="42" t="inlineStr">
-        <is>
-          <t>MH</t>
-        </is>
-      </c>
-      <c r="D20" s="42" t="inlineStr">
-        <is>
-          <t>E04/E08</t>
-        </is>
-      </c>
-      <c r="E20" s="42" t="inlineStr">
-        <is>
-          <t>ex J-BASSIN-OUEST</t>
-        </is>
-      </c>
+      <c r="A20" s="42" t="n"/>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="42" t="n"/>
+      <c r="E20" s="42" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="42" t="inlineStr">
-        <is>
-          <t>Ouest P-W1…P-W6</t>
-        </is>
-      </c>
-      <c r="B21" s="42" t="inlineStr">
-        <is>
-          <t>P-W1…P-W6</t>
-        </is>
-      </c>
-      <c r="C21" s="42" t="inlineStr">
-        <is>
-          <t>CB/MH</t>
-        </is>
-      </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>E05A…E05E,E04</t>
-        </is>
-      </c>
-      <c r="E21" s="42" t="inlineStr">
-        <is>
-          <t>Bande ouest (leaders plan peu lisibles)</t>
-        </is>
-      </c>
+      <c r="A21" s="42" t="n"/>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="42" t="n"/>
+      <c r="D21" s="42" t="n"/>
+      <c r="E21" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fix Noeuds V_required: use buffer time, not Note column
V_required was K*J*60 while J held text notes (#VALUE!). Restore
t_buffer in J from Inputs!B23; improve Qin for From_Node catchbasins.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
+++ b/engineering/drainage-design/Reseau_tresfond_hybride_retention_07_08.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="165" formatCode="[&lt;1]0.000;0.00"/>
     <numFmt numFmtId="166" formatCode="[&lt;1]0.0000;0.000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -90,6 +90,10 @@
     <font>
       <b val="1"/>
       <color rgb="001B4F72"/>
+    </font>
+    <font>
+      <color rgb="00922B21"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="15">
@@ -224,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -300,6 +304,10 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -33803,7 +33811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M204"/>
+  <dimension ref="A1:N204"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="17.28515625" customWidth="1" style="22" min="1" max="1"/>
@@ -33814,7 +33822,9 @@
     <col width="12" customWidth="1" style="22" min="7" max="7"/>
     <col width="13" customWidth="1" style="22" min="8" max="8"/>
     <col width="12" customWidth="1" style="22" min="9" max="12"/>
+    <col width="12" customWidth="1" style="22" min="10" max="10"/>
     <col width="10" customWidth="1" style="22" min="13" max="13"/>
+    <col width="45" customWidth="1" style="22" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -33824,6 +33834,13 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="36" customHeight="1" s="22">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t>V_required = Qin_peak × t_buffer × 60. t_buffer = Inputs!B23 (pas la colonne Note). Qin = débits arrivant (To_Node) + Q_local des éléments partant de ce noeud (From_Node).</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="29.25" customHeight="1" s="22">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -33872,22 +33889,27 @@
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
+          <t>t_buffer_min</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Qin_peak_m3s</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>V_required_m3</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Node_check</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Note</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>Qin_peak_m3s</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>V_required_m3</t>
-        </is>
-      </c>
-      <c r="M3" s="7" t="inlineStr">
-        <is>
-          <t>Node_check</t>
         </is>
       </c>
     </row>
@@ -33923,25 +33945,29 @@
       </c>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="10">
-        <f>IF(A4="","",IF(UPPER(TRIM(F4))="CIRC",PI()*(G4/2)^2*E4,IF(UPPER(TRIM(F4))="RECT",G4*H4*E4,"")))</f>
-        <v/>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
+        <f>IF(A4="","",IF(OR(E4="",G4=""),"",IF(UPPER(TRIM(F4))="CIRC",PI()*(G4/2)^2*E4,IF(UPPER(TRIM(F4))="RECT",IF(H4="","",G4*H4*E4),""))))</f>
+        <v/>
+      </c>
+      <c r="J4" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K4" s="10">
+        <f>IF(A4="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A4)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A4))</f>
+        <v/>
+      </c>
+      <c r="L4" s="52">
+        <f>IF(OR(A4="",K4=""),"",K4*J4*60)</f>
+        <v/>
+      </c>
+      <c r="M4" s="3">
+        <f>IF(A4="","",IF(OR(I4="",L4=""),"INFO",IF(I4&gt;=L4,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>CB ouest — reçoit gazon+pavé ouest</t>
         </is>
-      </c>
-      <c r="K4" s="10">
-        <f>IF(A4="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A4))</f>
-        <v/>
-      </c>
-      <c r="L4" s="10">
-        <f>IF(OR(K4="",J4=""),"",K4*J4*60)</f>
-        <v/>
-      </c>
-      <c r="M4" s="3">
-        <f>IF(A4="","",IF(OR(I4="",L4=""),"",IF(I4&gt;=L4,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="5">
@@ -33975,25 +34001,29 @@
       </c>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="10">
-        <f>IF(A5="","",IF(UPPER(TRIM(F5))="CIRC",PI()*(G5/2)^2*E5,IF(UPPER(TRIM(F5))="RECT",G5*H5*E5,"")))</f>
-        <v/>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
+        <f>IF(A5="","",IF(OR(E5="",G5=""),"",IF(UPPER(TRIM(F5))="CIRC",PI()*(G5/2)^2*E5,IF(UPPER(TRIM(F5))="RECT",IF(H5="","",G5*H5*E5),""))))</f>
+        <v/>
+      </c>
+      <c r="J5" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K5" s="10">
+        <f>IF(A5="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A5)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A5))</f>
+        <v/>
+      </c>
+      <c r="L5" s="52">
+        <f>IF(OR(A5="",K5=""),"",K5*J5*60)</f>
+        <v/>
+      </c>
+      <c r="M5" s="3">
+        <f>IF(A5="","",IF(OR(I5="",L5=""),"INFO",IF(I5&gt;=L5,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>CB est sud — reçoit bande arbres + sud-est</t>
         </is>
-      </c>
-      <c r="K5" s="10">
-        <f>IF(A5="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A5))</f>
-        <v/>
-      </c>
-      <c r="L5" s="10">
-        <f>IF(OR(K5="",J5=""),"",K5*J5*60)</f>
-        <v/>
-      </c>
-      <c r="M5" s="3">
-        <f>IF(A5="","",IF(OR(I5="",L5=""),"",IF(I5&gt;=L5,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -34027,25 +34057,29 @@
       </c>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="10">
-        <f>IF(A6="","",IF(UPPER(TRIM(F6))="CIRC",PI()*(G6/2)^2*E6,IF(UPPER(TRIM(F6))="RECT",G6*H6*E6,"")))</f>
-        <v/>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
+        <f>IF(A6="","",IF(OR(E6="",G6=""),"",IF(UPPER(TRIM(F6))="CIRC",PI()*(G6/2)^2*E6,IF(UPPER(TRIM(F6))="RECT",IF(H6="","",G6*H6*E6),""))))</f>
+        <v/>
+      </c>
+      <c r="J6" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K6" s="10">
+        <f>IF(A6="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A6)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A6))</f>
+        <v/>
+      </c>
+      <c r="L6" s="52">
+        <f>IF(OR(A6="",K6=""),"",K6*J6*60)</f>
+        <v/>
+      </c>
+      <c r="M6" s="3">
+        <f>IF(A6="","",IF(OR(I6="",L6=""),"INFO",IF(I6&gt;=L6,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>Regard — fusion ouest+est vers rue</t>
         </is>
-      </c>
-      <c r="K6" s="10">
-        <f>IF(A6="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A6))</f>
-        <v/>
-      </c>
-      <c r="L6" s="10">
-        <f>IF(OR(K6="",J6=""),"",K6*J6*60)</f>
-        <v/>
-      </c>
-      <c r="M6" s="3">
-        <f>IF(A6="","",IF(OR(I6="",L6=""),"",IF(I6&gt;=L6,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="7">
@@ -34075,25 +34109,29 @@
       </c>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="10">
-        <f>IF(A7="","",IF(UPPER(TRIM(F7))="CIRC",PI()*(G7/2)^2*E7,IF(UPPER(TRIM(F7))="RECT",G7*H7*E7,"")))</f>
-        <v/>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>Réseau pluvial existant (rue)</t>
-        </is>
+        <f>IF(A7="","",IF(OR(E7="",G7=""),"",IF(UPPER(TRIM(F7))="CIRC",PI()*(G7/2)^2*E7,IF(UPPER(TRIM(F7))="RECT",IF(H7="","",G7*H7*E7),""))))</f>
+        <v/>
+      </c>
+      <c r="J7" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
       </c>
       <c r="K7" s="10">
-        <f>IF(A7="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A7))</f>
-        <v/>
-      </c>
-      <c r="L7" s="10">
-        <f>IF(OR(K7="",J7=""),"",K7*J7*60)</f>
+        <f>IF(A7="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A7)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="52">
+        <f>IF(A7="","","n/a")</f>
         <v/>
       </c>
       <c r="M7" s="3">
-        <f>IF(A7="","",IF(OR(I7="",L7=""),"",IF(I7&gt;=L7,"OK","CHECK")))</f>
-        <v/>
+        <f>IF(A7="","","N/A (existant)")</f>
+        <v/>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Réseau existant (rue) — pas de volume de stockage à vérifier</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -34128,25 +34166,29 @@
       </c>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="10">
-        <f>IF(A8="","",IF(UPPER(TRIM(F8))="CIRC",PI()*(G8/2)^2*E8,IF(UPPER(TRIM(F8))="RECT",G8*H8*E8,"")))</f>
-        <v/>
-      </c>
-      <c r="J8" s="8" t="inlineStr">
+        <f>IF(A8="","",IF(OR(E8="",G8=""),"",IF(UPPER(TRIM(F8))="CIRC",PI()*(G8/2)^2*E8,IF(UPPER(TRIM(F8))="RECT",IF(H8="","",G8*H8*E8),""))))</f>
+        <v/>
+      </c>
+      <c r="J8" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K8" s="10">
+        <f>IF(A8="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A8)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A8))</f>
+        <v/>
+      </c>
+      <c r="L8" s="52">
+        <f>IF(OR(A8="",K8=""),"",K8*J8*60)</f>
+        <v/>
+      </c>
+      <c r="M8" s="3">
+        <f>IF(A8="","",IF(OR(I8="",L8=""),"INFO",IF(I8&gt;=L8,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>Sortie mécanique bâtiment (toit/tréfond)</t>
         </is>
-      </c>
-      <c r="K8" s="10">
-        <f>IF(A8="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A8))</f>
-        <v/>
-      </c>
-      <c r="L8" s="10">
-        <f>IF(OR(K8="",J8=""),"",K8*J8*60)</f>
-        <v/>
-      </c>
-      <c r="M8" s="3">
-        <f>IF(A8="","",IF(OR(I8="",L8=""),"",IF(I8&gt;=L8,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="9">
@@ -34184,25 +34226,29 @@
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(A9="","",IF(UPPER(TRIM(F9))="CIRC",PI()*(G9/2)^2*E9,IF(UPPER(TRIM(F9))="RECT",G9*H9*E9,"")))</f>
-        <v/>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
+        <f>IF(A9="","",IF(OR(E9="",G9=""),"",IF(UPPER(TRIM(F9))="CIRC",PI()*(G9/2)^2*E9,IF(UPPER(TRIM(F9))="RECT",IF(H9="","",G9*H9*E9),""))))</f>
+        <v/>
+      </c>
+      <c r="J9" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K9" s="10">
+        <f>IF(A9="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A9)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A9))</f>
+        <v/>
+      </c>
+      <c r="L9" s="52">
+        <f>IF(OR(A9="",K9=""),"",K9*J9*60)</f>
+        <v/>
+      </c>
+      <c r="M9" s="3">
+        <f>IF(A9="","",IF(OR(I9="",L9=""),"INFO",IF(I9&gt;=L9,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>Bassin rétention EZ-STORM</t>
         </is>
-      </c>
-      <c r="K9" s="10">
-        <f>IF(A9="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A9))</f>
-        <v/>
-      </c>
-      <c r="L9" s="10">
-        <f>IF(OR(K9="",J9=""),"",K9*J9*60)</f>
-        <v/>
-      </c>
-      <c r="M9" s="3">
-        <f>IF(A9="","",IF(OR(I9="",L9=""),"",IF(I9&gt;=L9,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="10">
@@ -34239,25 +34285,29 @@
         <v>20</v>
       </c>
       <c r="I10" s="10">
-        <f>IF(A10="","",IF(UPPER(TRIM(F10))="CIRC",PI()*(G10/2)^2*E10,IF(UPPER(TRIM(F10))="RECT",G10*H10*E10,"")))</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="inlineStr">
+        <f>IF(A10="","",IF(OR(E10="",G10=""),"",IF(UPPER(TRIM(F10))="CIRC",PI()*(G10/2)^2*E10,IF(UPPER(TRIM(F10))="RECT",IF(H10="","",G10*H10*E10),""))))</f>
+        <v/>
+      </c>
+      <c r="J10" s="52">
+        <f>Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="K10" s="10">
+        <f>IF(A10="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A10)+SUMIFS(Elements_hybrides!$O:$O,Elements_hybrides!$C:$C,$A10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="52">
+        <f>IF(OR(A10="",K10=""),"",K10*J10*60)</f>
+        <v/>
+      </c>
+      <c r="M10" s="3">
+        <f>IF(A10="","",IF(OR(I10="",L10=""),"INFO",IF(I10&gt;=L10,"OK","CHECK")))</f>
+        <v/>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>Noeud conceptuel bande arbres (pas de CB)</t>
         </is>
-      </c>
-      <c r="K10" s="10">
-        <f>IF(A10="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A10))</f>
-        <v/>
-      </c>
-      <c r="L10" s="10">
-        <f>IF(OR(K10="",J10=""),"",K10*J10*60)</f>
-        <v/>
-      </c>
-      <c r="M10" s="3">
-        <f>IF(A10="","",IF(OR(I10="",L10=""),"",IF(I10&gt;=L10,"OK","CHECK")))</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -34276,22 +34326,10 @@
         <f>IF(A11="","",IF(UPPER(TRIM(F11))="CIRC",PI()*(G11/2)^2*E11,IF(UPPER(TRIM(F11))="RECT",G11*H11*E11,"")))</f>
         <v/>
       </c>
-      <c r="J11" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K11" s="10">
-        <f>IF(A11="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A11))</f>
-        <v/>
-      </c>
-      <c r="L11" s="10">
-        <f>IF(OR(K11="",J11=""),"",K11*J11*60)</f>
-        <v/>
-      </c>
-      <c r="M11" s="3">
-        <f>IF(A11="","",IF(OR(I11="",L11=""),"",IF(I11&gt;=L11,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="10" t="n"/>
+      <c r="L11" s="10" t="n"/>
+      <c r="M11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -34309,22 +34347,10 @@
         <f>IF(A12="","",IF(UPPER(TRIM(F12))="CIRC",PI()*(G12/2)^2*E12,IF(UPPER(TRIM(F12))="RECT",G12*H12*E12,"")))</f>
         <v/>
       </c>
-      <c r="J12" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K12" s="10">
-        <f>IF(A12="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A12))</f>
-        <v/>
-      </c>
-      <c r="L12" s="10">
-        <f>IF(OR(K12="",J12=""),"",K12*J12*60)</f>
-        <v/>
-      </c>
-      <c r="M12" s="3">
-        <f>IF(A12="","",IF(OR(I12="",L12=""),"",IF(I12&gt;=L12,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J12" s="8" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -34342,22 +34368,10 @@
         <f>IF(A13="","",IF(UPPER(TRIM(F13))="CIRC",PI()*(G13/2)^2*E13,IF(UPPER(TRIM(F13))="RECT",G13*H13*E13,"")))</f>
         <v/>
       </c>
-      <c r="J13" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K13" s="10">
-        <f>IF(A13="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A13))</f>
-        <v/>
-      </c>
-      <c r="L13" s="10">
-        <f>IF(OR(K13="",J13=""),"",K13*J13*60)</f>
-        <v/>
-      </c>
-      <c r="M13" s="3">
-        <f>IF(A13="","",IF(OR(I13="",L13=""),"",IF(I13&gt;=L13,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="10" t="n"/>
+      <c r="L13" s="10" t="n"/>
+      <c r="M13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -34375,22 +34389,10 @@
         <f>IF(A14="","",IF(UPPER(TRIM(F14))="CIRC",PI()*(G14/2)^2*E14,IF(UPPER(TRIM(F14))="RECT",G14*H14*E14,"")))</f>
         <v/>
       </c>
-      <c r="J14" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K14" s="10">
-        <f>IF(A14="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A14))</f>
-        <v/>
-      </c>
-      <c r="L14" s="10">
-        <f>IF(OR(K14="",J14=""),"",K14*J14*60)</f>
-        <v/>
-      </c>
-      <c r="M14" s="3">
-        <f>IF(A14="","",IF(OR(I14="",L14=""),"",IF(I14&gt;=L14,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J14" s="8" t="n"/>
+      <c r="K14" s="10" t="n"/>
+      <c r="L14" s="10" t="n"/>
+      <c r="M14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -34408,22 +34410,10 @@
         <f>IF(A15="","",IF(UPPER(TRIM(F15))="CIRC",PI()*(G15/2)^2*E15,IF(UPPER(TRIM(F15))="RECT",G15*H15*E15,"")))</f>
         <v/>
       </c>
-      <c r="J15" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K15" s="10">
-        <f>IF(A15="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A15))</f>
-        <v/>
-      </c>
-      <c r="L15" s="10">
-        <f>IF(OR(K15="",J15=""),"",K15*J15*60)</f>
-        <v/>
-      </c>
-      <c r="M15" s="3">
-        <f>IF(A15="","",IF(OR(I15="",L15=""),"",IF(I15&gt;=L15,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="10" t="n"/>
+      <c r="L15" s="10" t="n"/>
+      <c r="M15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -34441,21 +34431,10 @@
         <f>IF(A16="","",IF(UPPER(TRIM(F16))="CIRC",PI()*(G16/2)^2*E16,IF(UPPER(TRIM(F16))="RECT",G16*H16*E16,"")))</f>
         <v/>
       </c>
-      <c r="J16" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="K16" s="10">
-        <f>IF(A16="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A16))</f>
-        <v/>
-      </c>
-      <c r="L16" s="10">
-        <f>IF(OR(K16="",J16=""),"",K16*J16*60)</f>
-        <v/>
-      </c>
-      <c r="M16" s="3">
-        <f>IF(A16="","",IF(OR(I16="",L16=""),"",IF(I16&gt;=L16,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="10" t="n"/>
+      <c r="L16" s="10" t="n"/>
+      <c r="M16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -34473,22 +34452,10 @@
         <f>IF(A17="","",IF(UPPER(TRIM(F17))="CIRC",PI()*(G17/2)^2*E17,IF(UPPER(TRIM(F17))="RECT",G17*H17*E17,"")))</f>
         <v/>
       </c>
-      <c r="J17" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K17" s="10">
-        <f>IF(A17="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A17))</f>
-        <v/>
-      </c>
-      <c r="L17" s="10">
-        <f>IF(OR(K17="",J17=""),"",K17*J17*60)</f>
-        <v/>
-      </c>
-      <c r="M17" s="3">
-        <f>IF(A17="","",IF(OR(I17="",L17=""),"",IF(I17&gt;=L17,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="10" t="n"/>
+      <c r="L17" s="10" t="n"/>
+      <c r="M17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -34506,22 +34473,10 @@
         <f>IF(A18="","",IF(UPPER(TRIM(F18))="CIRC",PI()*(G18/2)^2*E18,IF(UPPER(TRIM(F18))="RECT",G18*H18*E18,"")))</f>
         <v/>
       </c>
-      <c r="J18" s="8">
-        <f>Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="K18" s="10">
-        <f>IF(A18="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A18))</f>
-        <v/>
-      </c>
-      <c r="L18" s="10">
-        <f>IF(OR(K18="",J18=""),"",K18*J18*60)</f>
-        <v/>
-      </c>
-      <c r="M18" s="3">
-        <f>IF(A18="","",IF(OR(I18="",L18=""),"",IF(I18&gt;=L18,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="J18" s="8" t="n"/>
+      <c r="K18" s="10" t="n"/>
+      <c r="L18" s="10" t="n"/>
+      <c r="M18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -34540,18 +34495,9 @@
         <v/>
       </c>
       <c r="J19" s="8" t="n"/>
-      <c r="K19" s="10">
-        <f>IF(A19="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A19))</f>
-        <v/>
-      </c>
-      <c r="L19" s="10">
-        <f>IF(OR(K19="",J19=""),"",K19*J19*60)</f>
-        <v/>
-      </c>
-      <c r="M19" s="3">
-        <f>IF(A19="","",IF(OR(I19="",L19=""),"",IF(I19&gt;=L19,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K19" s="10" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -34570,18 +34516,9 @@
         <v/>
       </c>
       <c r="J20" s="8" t="n"/>
-      <c r="K20" s="10">
-        <f>IF(A20="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A20))</f>
-        <v/>
-      </c>
-      <c r="L20" s="10">
-        <f>IF(OR(K20="",J20=""),"",K20*J20*60)</f>
-        <v/>
-      </c>
-      <c r="M20" s="3">
-        <f>IF(A20="","",IF(OR(I20="",L20=""),"",IF(I20&gt;=L20,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="10" t="n"/>
+      <c r="M20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -34600,18 +34537,9 @@
         <v/>
       </c>
       <c r="J21" s="8" t="n"/>
-      <c r="K21" s="10">
-        <f>IF(A21="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A21))</f>
-        <v/>
-      </c>
-      <c r="L21" s="10">
-        <f>IF(OR(K21="",J21=""),"",K21*J21*60)</f>
-        <v/>
-      </c>
-      <c r="M21" s="3">
-        <f>IF(A21="","",IF(OR(I21="",L21=""),"",IF(I21&gt;=L21,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K21" s="10" t="n"/>
+      <c r="L21" s="10" t="n"/>
+      <c r="M21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -34630,18 +34558,9 @@
         <v/>
       </c>
       <c r="J22" s="8" t="n"/>
-      <c r="K22" s="10">
-        <f>IF(A22="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A22))</f>
-        <v/>
-      </c>
-      <c r="L22" s="10">
-        <f>IF(OR(K22="",J22=""),"",K22*J22*60)</f>
-        <v/>
-      </c>
-      <c r="M22" s="3">
-        <f>IF(A22="","",IF(OR(I22="",L22=""),"",IF(I22&gt;=L22,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="10" t="n"/>
+      <c r="M22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -34660,18 +34579,9 @@
         <v/>
       </c>
       <c r="J23" s="8" t="n"/>
-      <c r="K23" s="10">
-        <f>IF(A23="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A23))</f>
-        <v/>
-      </c>
-      <c r="L23" s="10">
-        <f>IF(OR(K23="",J23=""),"",K23*J23*60)</f>
-        <v/>
-      </c>
-      <c r="M23" s="3">
-        <f>IF(A23="","",IF(OR(I23="",L23=""),"",IF(I23&gt;=L23,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K23" s="10" t="n"/>
+      <c r="L23" s="10" t="n"/>
+      <c r="M23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -34690,18 +34600,9 @@
         <v/>
       </c>
       <c r="J24" s="8" t="n"/>
-      <c r="K24" s="10">
-        <f>IF(A24="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A24))</f>
-        <v/>
-      </c>
-      <c r="L24" s="10">
-        <f>IF(OR(K24="",J24=""),"",K24*J24*60)</f>
-        <v/>
-      </c>
-      <c r="M24" s="3">
-        <f>IF(A24="","",IF(OR(I24="",L24=""),"",IF(I24&gt;=L24,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K24" s="10" t="n"/>
+      <c r="L24" s="10" t="n"/>
+      <c r="M24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -34720,18 +34621,9 @@
         <v/>
       </c>
       <c r="J25" s="8" t="n"/>
-      <c r="K25" s="10">
-        <f>IF(A25="","",SUMIFS(Elements_hybrides!$Q:$Q,Elements_hybrides!$D:$D,$A25))</f>
-        <v/>
-      </c>
-      <c r="L25" s="10">
-        <f>IF(OR(K25="",J25=""),"",K25*J25*60)</f>
-        <v/>
-      </c>
-      <c r="M25" s="3">
-        <f>IF(A25="","",IF(OR(I25="",L25=""),"",IF(I25&gt;=L25,"OK","CHECK")))</f>
-        <v/>
-      </c>
+      <c r="K25" s="10" t="n"/>
+      <c r="L25" s="10" t="n"/>
+      <c r="M25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>

</xml_diff>